<commit_message>
🔄 Actualización automática del mapa (2025-10-14 08:04:19)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -1480,7 +1480,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>AYKO</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>Sin Asignar</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>AYKO</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sin Asignar</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -5271,7 +5271,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5451,27 +5451,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4680</t>
+          <t>4082</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1/22/2025</t>
+          <t>12/21/2024</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CUENCA 3345</t>
+          <t>MERCEDES 254</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>801901755</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Colocar R200 para pedir traspaso de equipo</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -5508,14 +5508,14 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>-58.496935</v>
+        <v>-58.484232</v>
       </c>
       <c r="N3" t="n">
-        <v>-34.599084</v>
+        <v>-34.631431</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -5525,39 +5525,39 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>4680</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>1/22/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>CUENCA 3345</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>802843289</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -5594,24 +5594,24 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>-58.441405</v>
+        <v>-58.496935</v>
       </c>
       <c r="N4" t="n">
-        <v>-34.594348</v>
+        <v>-34.599084</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -5623,7 +5623,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5633,17 +5633,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>804309801</t>
+          <t>804309655</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -5656,7 +5656,11 @@
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+        </is>
+      </c>
       <c r="I5" t="n">
         <v>1</v>
       </c>
@@ -5676,14 +5680,14 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>-58.483821</v>
+        <v>-58.441405</v>
       </c>
       <c r="N5" t="n">
-        <v>-34.677698</v>
+        <v>-34.594348</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -5693,7 +5697,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -5705,27 +5709,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>-440</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>5/26/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LAPRIDA 1374</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>807005369</t>
+          <t>804309801</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5738,51 +5742,215 @@
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Se coloco columna nueva queda pendiente de traspaso</t>
-        </is>
-      </c>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="M6" t="n">
+        <v>-58.483821</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-34.677698</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>PAV-Q</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6284</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>6/30/2025</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CHILE 2561</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>807851584</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="M7" t="n">
+        <v>-58.401827</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-34.617667</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>CEN-M</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>5999</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>8/12/2025</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MARMOL, JOSE 228</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>808918687</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Cambio</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="M6" t="n">
-        <v>-58.406585</v>
-      </c>
-      <c r="N6" t="n">
-        <v>-34.592933</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Recoleta</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
+      <c r="M8" t="n">
+        <v>-58.425858</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-34.61629</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>AGU-B</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>ALM-D</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -5799,7 +5967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5979,27 +6147,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12/21/2024</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MERCEDES 254</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -6014,7 +6182,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Colocar R200 para pedir traspaso de equipo</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -6036,14 +6204,14 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>-58.484232</v>
+        <v>-58.451835</v>
       </c>
       <c r="N3" t="n">
-        <v>-34.631431</v>
+        <v>-34.562646</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -6053,178 +6221,10 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
-        <is>
-          <t>ARATO-25058.PO.2DEV</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>-405</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>5/8/2025</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Arcos 1855</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>805791908</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>AYKO</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="M4" t="n">
-        <v>-58.451835</v>
-      </c>
-      <c r="N4" t="n">
-        <v>-34.562646</v>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>BLO-N</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>6284</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>6/30/2025</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>CHILE 2561</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>807851584</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>AYKO</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="M5" t="n">
-        <v>-58.401827</v>
-      </c>
-      <c r="N5" t="n">
-        <v>-34.617667</v>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>CEN-M</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -6339,27 +6339,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>-440</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>5/26/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>LAPRIDA 1374</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>807005369</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -6374,7 +6374,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+          <t>Se coloco columna nueva queda pendiente de traspaso</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -6387,7 +6387,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -6396,14 +6396,14 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>-58.425858</v>
+        <v>-58.406585</v>
       </c>
       <c r="N2" t="n">
-        <v>-34.61629</v>
+        <v>-34.592933</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -6413,7 +6413,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>AGU-B</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-25 10:26:30)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2376,22 +2376,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>-317</t>
+          <t>5657</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4/9/2025</t>
+          <t>4/23/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ /ALT/ 612</t>
+          <t>COCHABAMBA 2207</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2406,12 +2406,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>804569034</t>
+          <t>804903806</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Terminar traspaso, retirar columna</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2430,17 +2430,17 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.445131</v>
+        <v>-58.396135</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.572117</v>
+        <v>-34.624285</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>COG-C</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2462,17 +2462,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5657</t>
+          <t>5682</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4/23/2025</t>
+          <t>4/29/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COCHABAMBA 2207</t>
+          <t>República Bolivariana de Venezuela 2701</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2492,12 +2492,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>805507294</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2507,26 +2507,26 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.396135</v>
+        <v>-58.404913</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.624285</v>
+        <v>-34.615857</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2536,7 +2536,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2548,22 +2548,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5682</t>
+          <t>5708</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>República Bolivariana de Venezuela 2701</t>
+          <t>SARMIENTO 1741</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2578,12 +2578,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>805507294</t>
+          <t>805579089</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Pendiente de traspaso nodo y fuente</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2593,26 +2593,26 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.404913</v>
+        <v>-58.391419</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.615857</v>
+        <v>-34.605543</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2622,7 +2622,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CEN-E</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2634,17 +2634,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5686</t>
+          <t>5731</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HUMBERTO 1° 1999</t>
+          <t>RIOBAMBA 659</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2664,12 +2664,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>805507324</t>
+          <t>805579188</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso fuente</t>
+          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2691,14 +2691,14 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.394304</v>
+        <v>-58.394118</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.621645</v>
+        <v>-34.601416</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -2708,7 +2708,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>CEN-B</t>
+          <t>RET-H</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2720,22 +2720,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2750,12 +2750,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>805579089</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2777,24 +2777,24 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.391419</v>
+        <v>-58.451835</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.605543</v>
+        <v>-34.562646</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>CEN-E</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2806,22 +2806,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5731</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>RIOBAMBA 659</t>
+          <t>MAZA 181</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2836,12 +2836,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>807215439</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2863,10 +2863,10 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.394118</v>
+        <v>-58.416477</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.601416</v>
+        <v>-34.61303</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2880,7 +2880,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>CLI-I</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2892,22 +2892,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>6076</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>MATHEU 727</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2922,14 +2922,10 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>805791908</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
-        </is>
-      </c>
+          <t>ICD31456940</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2937,7 +2933,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2949,24 +2945,24 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.451835</v>
+        <v>-58.400169</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.562646</v>
+        <v>-34.617784</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>CEN-N</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2978,22 +2974,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>-440</t>
+          <t>6284</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>5/26/2025</t>
+          <t>6/30/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LAPRIDA 1374</t>
+          <t>CHILE 2561</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3008,14 +3004,10 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>807005369</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Se coloco columna nueva queda pendiente de traspaso</t>
-        </is>
-      </c>
+          <t>807851584</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -3032,17 +3024,17 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.406585</v>
+        <v>-58.401827</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.592933</v>
+        <v>-34.617667</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3052,7 +3044,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>AGU-B</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3064,17 +3056,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>5999</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>8/12/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MAZA 181</t>
+          <t>MARMOL, JOSE 228</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3094,12 +3086,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>807215439</t>
+          <t>808918687</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3109,7 +3101,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3118,13 +3110,13 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.416477</v>
+        <v>-58.425858</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.61303</v>
+        <v>-34.61629</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3138,7 +3130,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>CLI-I</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3150,22 +3142,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6076</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MATHEU 727</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3180,10 +3172,14 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>ICD30508311</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -3191,26 +3187,26 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Nodo TLC</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.400169</v>
+        <v>-58.435017</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.617784</v>
+        <v>-34.622044</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -3220,7 +3216,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>CEN-N</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3232,22 +3228,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6284</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6/30/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CHILE 2561</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3262,10 +3258,14 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>807851584</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
+          <t>ICD30593982</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -3278,21 +3278,21 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.401827</v>
+        <v>-58.443232</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.617667</v>
+        <v>-34.620007</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3314,22 +3314,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3344,12 +3344,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>809910087</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3359,7 +3359,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3368,17 +3368,17 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.425858</v>
+        <v>-58.442045</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.61629</v>
+        <v>-34.594303</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3400,22 +3400,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>7570</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>10/6/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3430,12 +3430,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>Colocar R150 o R200</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3445,22 +3445,22 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.435017</v>
+        <v>-58.465176</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.622044</v>
+        <v>-34.680979</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3474,7 +3474,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3486,22 +3486,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3516,12 +3516,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3536,31 +3536,31 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.443232</v>
+        <v>-58.444996</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.620007</v>
+        <v>-34.564443</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3572,22 +3572,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3602,12 +3602,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3626,17 +3626,17 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.442045</v>
+        <v>-58.4018</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.594303</v>
+        <v>-34.590471</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3646,7 +3646,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3658,22 +3658,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3688,12 +3688,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Colocar R150 o R200</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3703,26 +3703,26 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.465176</v>
+        <v>-58.436262</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.680979</v>
+        <v>-34.600478</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3744,22 +3744,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>-649</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10/23/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Arribeños 1438</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3774,12 +3774,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3798,17 +3798,17 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.444996</v>
+        <v>-58.510994</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.564443</v>
+        <v>-34.655027</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -3818,7 +3818,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>BLO-K</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3830,22 +3830,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5749</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
+          <t>LAMBARE 864</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3860,12 +3860,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>811453866</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -3884,17 +3884,17 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.4018</v>
+        <v>-58.430579</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.590471</v>
+        <v>-34.604908</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -3904,7 +3904,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>ALM-M</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -3916,22 +3916,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S01150217</t>
+          <t>3875</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Vera 311</t>
+          <t>Castelli 60</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -3946,41 +3946,29 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>01230602</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Traspasar Fuente</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Fuente Teco</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
+          <t>traspaso propio tlc coloco columna</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.436262</v>
+        <v>-58.404691</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.600478</v>
+        <v>-34.609194</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -3990,256 +3978,10 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>-670</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>11/10/2025</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Timoteo Gordillo 1666</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>810651269</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L43" t="n">
-        <v>1</v>
-      </c>
-      <c r="M43" t="n">
-        <v>-58.510994</v>
-      </c>
-      <c r="N43" t="n">
-        <v>-34.655027</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>PAV-J</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>8043</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>1/8/2026</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>LAMBARE 864</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>811453866</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>corroida</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L44" t="n">
-        <v>1</v>
-      </c>
-      <c r="M44" t="n">
-        <v>-58.430579</v>
-      </c>
-      <c r="N44" t="n">
-        <v>-34.604908</v>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>ALM-M</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>3875</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>1/16/2026</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Castelli 60</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>traspaso propio tlc coloco columna</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="n">
-        <v>1</v>
-      </c>
-      <c r="M45" t="n">
-        <v>-58.404691</v>
-      </c>
-      <c r="N45" t="n">
-        <v>-34.609194</v>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>CLI-D</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -4256,7 +3998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6218,22 +5960,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>-317</t>
+          <t>5657</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4/9/2025</t>
+          <t>4/23/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ /ALT/ 612</t>
+          <t>COCHABAMBA 2207</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -6248,12 +5990,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>804569034</t>
+          <t>804903806</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Terminar traspaso, retirar columna</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -6263,7 +6005,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -6272,17 +6014,17 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.445131</v>
+        <v>-58.396135</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.572117</v>
+        <v>-34.624285</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -6292,7 +6034,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>COG-C</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -6304,17 +6046,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5657</t>
+          <t>5682</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4/23/2025</t>
+          <t>4/29/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>COCHABAMBA 2207</t>
+          <t>República Bolivariana de Venezuela 2701</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -6334,12 +6076,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>805507294</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -6349,26 +6091,26 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.396135</v>
+        <v>-58.404913</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.624285</v>
+        <v>-34.615857</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -6378,7 +6120,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -6390,22 +6132,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5682</t>
+          <t>5708</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>República Bolivariana de Venezuela 2701</t>
+          <t>SARMIENTO 1741</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6420,12 +6162,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>805507294</t>
+          <t>805579089</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Pendiente de traspaso nodo y fuente</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -6435,26 +6177,26 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L26" t="n">
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.404913</v>
+        <v>-58.391419</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.615857</v>
+        <v>-34.605543</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -6464,7 +6206,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CEN-E</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -6476,17 +6218,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5686</t>
+          <t>5731</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>HUMBERTO 1° 1999</t>
+          <t>RIOBAMBA 659</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -6506,12 +6248,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>805507324</t>
+          <t>805579188</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso fuente</t>
+          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -6521,7 +6263,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -6533,14 +6275,14 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.394304</v>
+        <v>-58.394118</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.621645</v>
+        <v>-34.601416</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
@@ -6550,7 +6292,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>CEN-B</t>
+          <t>RET-H</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -6562,22 +6304,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -6592,12 +6334,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>805579089</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -6607,7 +6349,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -6619,24 +6361,24 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.391419</v>
+        <v>-58.451835</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.605543</v>
+        <v>-34.562646</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>CEN-E</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -6648,22 +6390,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5731</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>RIOBAMBA 659</t>
+          <t>MAZA 181</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6678,12 +6420,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>807215439</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -6705,10 +6447,10 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.394118</v>
+        <v>-58.416477</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.601416</v>
+        <v>-34.61303</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -6722,7 +6464,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>CLI-I</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -6734,22 +6476,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>6076</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>MATHEU 727</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -6764,14 +6506,10 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>805791908</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
-        </is>
-      </c>
+          <t>ICD31456940</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -6779,7 +6517,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -6791,24 +6529,24 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.451835</v>
+        <v>-58.400169</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.562646</v>
+        <v>-34.617784</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>CEN-N</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -6820,22 +6558,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>-440</t>
+          <t>6284</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>5/26/2025</t>
+          <t>6/30/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LAPRIDA 1374</t>
+          <t>CHILE 2561</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -6850,14 +6588,10 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>807005369</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Se coloco columna nueva queda pendiente de traspaso</t>
-        </is>
-      </c>
+          <t>807851584</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -6874,17 +6608,17 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.406585</v>
+        <v>-58.401827</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.592933</v>
+        <v>-34.617667</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -6894,7 +6628,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>AGU-B</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -6906,17 +6640,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>5999</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>8/12/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MAZA 181</t>
+          <t>MARMOL, JOSE 228</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6936,12 +6670,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>807215439</t>
+          <t>808918687</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -6951,7 +6685,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -6960,13 +6694,13 @@
         </is>
       </c>
       <c r="L32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.416477</v>
+        <v>-58.425858</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.61303</v>
+        <v>-34.61629</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -6980,7 +6714,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>CLI-I</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -6992,22 +6726,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6076</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MATHEU 727</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7022,10 +6756,14 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr"/>
+          <t>ICD30508311</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -7033,26 +6771,26 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Nodo TLC</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.400169</v>
+        <v>-58.435017</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.617784</v>
+        <v>-34.622044</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -7062,7 +6800,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>CEN-N</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -7074,22 +6812,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6284</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6/30/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CHILE 2561</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7104,10 +6842,14 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>807851584</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr"/>
+          <t>ICD30593982</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -7120,21 +6862,21 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.401827</v>
+        <v>-58.443232</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.617667</v>
+        <v>-34.620007</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -7144,7 +6886,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -7156,22 +6898,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7186,12 +6928,12 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>809910087</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -7201,7 +6943,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -7210,17 +6952,17 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.425858</v>
+        <v>-58.442045</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.61629</v>
+        <v>-34.594303</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -7230,7 +6972,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -7242,22 +6984,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>7570</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>10/6/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7272,12 +7014,12 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>Colocar R150 o R200</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -7287,22 +7029,22 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L36" t="n">
         <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.435017</v>
+        <v>-58.465176</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.622044</v>
+        <v>-34.680979</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -7316,7 +7058,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -7328,22 +7070,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7358,12 +7100,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -7378,31 +7120,31 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.443232</v>
+        <v>-58.444996</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.620007</v>
+        <v>-34.564443</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -7414,22 +7156,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7444,12 +7186,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -7468,17 +7210,17 @@
         </is>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.442045</v>
+        <v>-58.4018</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.594303</v>
+        <v>-34.590471</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -7488,7 +7230,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -7500,22 +7242,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7530,12 +7272,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Colocar R150 o R200</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -7545,26 +7287,26 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.465176</v>
+        <v>-58.436262</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.680979</v>
+        <v>-34.600478</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
@@ -7574,7 +7316,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -7586,22 +7328,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>-649</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>10/23/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Arribeños 1438</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -7616,12 +7358,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -7631,7 +7373,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -7640,17 +7382,17 @@
         </is>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.444996</v>
+        <v>-58.510994</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.564443</v>
+        <v>-34.655027</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
@@ -7660,7 +7402,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>BLO-K</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -7672,22 +7414,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5749</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
+          <t>LAMBARE 864</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -7702,12 +7444,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>811453866</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -7717,7 +7459,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -7726,17 +7468,17 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.4018</v>
+        <v>-58.430579</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.590471</v>
+        <v>-34.604908</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
@@ -7746,7 +7488,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>ALM-M</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -7758,22 +7500,22 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S01150217</t>
+          <t>3875</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Vera 311</t>
+          <t>Castelli 60</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -7788,41 +7530,29 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>01230602</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Traspasar Fuente</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>Fuente Teco</t>
-        </is>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
+          <t>traspaso propio tlc coloco columna</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
       <c r="L42" t="n">
         <v>1</v>
       </c>
       <c r="M42" t="n">
-        <v>-58.436262</v>
+        <v>-58.404691</v>
       </c>
       <c r="N42" t="n">
-        <v>-34.600478</v>
+        <v>-34.609194</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
@@ -7832,256 +7562,10 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R42" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>-670</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>11/10/2025</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Timoteo Gordillo 1666</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>810651269</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L43" t="n">
-        <v>1</v>
-      </c>
-      <c r="M43" t="n">
-        <v>-58.510994</v>
-      </c>
-      <c r="N43" t="n">
-        <v>-34.655027</v>
-      </c>
-      <c r="O43" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P43" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q43" t="inlineStr">
-        <is>
-          <t>PAV-J</t>
-        </is>
-      </c>
-      <c r="R43" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>8043</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>1/8/2026</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>LAMBARE 864</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>811453866</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>corroida</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L44" t="n">
-        <v>1</v>
-      </c>
-      <c r="M44" t="n">
-        <v>-58.430579</v>
-      </c>
-      <c r="N44" t="n">
-        <v>-34.604908</v>
-      </c>
-      <c r="O44" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P44" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q44" t="inlineStr">
-        <is>
-          <t>ALM-M</t>
-        </is>
-      </c>
-      <c r="R44" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>3875</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>1/16/2026</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>Castelli 60</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>traspaso propio tlc coloco columna</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr"/>
-      <c r="L45" t="n">
-        <v>1</v>
-      </c>
-      <c r="M45" t="n">
-        <v>-58.404691</v>
-      </c>
-      <c r="N45" t="n">
-        <v>-34.609194</v>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P45" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q45" t="inlineStr">
-        <is>
-          <t>CLI-D</t>
-        </is>
-      </c>
-      <c r="R45" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-28 12:28:51)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Propio" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Optical_Power" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3425,7 +3426,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3998,7 +3999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6984,22 +6985,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7019,7 +7020,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Colocar R150 o R200</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -7038,27 +7039,27 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.465176</v>
+        <v>-58.444996</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.680979</v>
+        <v>-34.564443</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -7070,22 +7071,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>-649</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10/23/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Arribeños 1438</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7100,12 +7101,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -7127,24 +7128,24 @@
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.444996</v>
+        <v>-58.4018</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.564443</v>
+        <v>-34.590471</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>BLO-K</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -7156,22 +7157,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5749</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7186,12 +7187,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -7201,26 +7202,26 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.4018</v>
+        <v>-58.436262</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.590471</v>
+        <v>-34.600478</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -7230,7 +7231,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -7242,22 +7243,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S01150217</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Vera 311</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7272,12 +7273,12 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>01230602</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Traspasar Fuente</t>
+          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -7287,36 +7288,36 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.436262</v>
+        <v>-58.510994</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.600478</v>
+        <v>-34.655027</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -7328,22 +7329,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>LAMBARE 864</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -7358,12 +7359,12 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>811453866</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -7385,24 +7386,24 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.510994</v>
+        <v>-58.430579</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.655027</v>
+        <v>-34.604908</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>ALM-M</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -7414,22 +7415,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8043</t>
+          <t>3875</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LAMBARE 864</t>
+          <t>Castelli 60</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -7444,37 +7445,25 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>811453866</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>corroida</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+          <t>traspaso propio tlc coloco columna</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="n">
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.430579</v>
+        <v>-58.404691</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.604908</v>
+        <v>-34.609194</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -7488,7 +7477,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>ALM-M</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
@@ -7497,75 +7486,193 @@
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>3875</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>1/16/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Castelli 60</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>F. De Reclamo</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Direccion</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Comuna</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Proveedor Asignado</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Observaciones</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Tipo de tarea</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Equipo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Tipo de Elemento</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Attachments</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Coordenada_X</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Coordenada_Y</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Operacion</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Zona</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>PD</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>7570</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>10/6/2025</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>Pendiente ADM</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>traspaso propio tlc coloco columna</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="n">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Colocar R150 o R200</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
         <v>1</v>
       </c>
-      <c r="M42" t="n">
-        <v>-58.404691</v>
-      </c>
-      <c r="N42" t="n">
-        <v>-34.609194</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
+      <c r="M2" t="n">
+        <v>-58.465176</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-34.680979</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>CLI-D</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-03-31 13:59:28)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -565,25 +565,21 @@
       <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="n">
-        <v>-58.395498</v>
-      </c>
-      <c r="N2" t="n">
-        <v>-34.59322</v>
-      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>No clasificado, consultar con mantenimiento</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>RET-B</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -4149,25 +4145,21 @@
       <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="n">
-        <v>-58.395498</v>
-      </c>
-      <c r="N2" t="n">
-        <v>-34.59322</v>
-      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>No clasificado, consultar con mantenimiento</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>RET-B</t>
+          <t>No ubicado</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-04-01 08:30:28)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -565,21 +565,25 @@
       <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>-58.395498</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-34.59322</v>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>No clasificado, consultar con mantenimiento</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>RET-B</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -4145,21 +4149,25 @@
       <c r="L2" t="n">
         <v>0</v>
       </c>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>-58.395498</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-34.59322</v>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>No clasificado, consultar con mantenimiento</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>No ubicado</t>
+          <t>RET-B</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-14 13:55:25)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="General" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Propio" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Optical_Power" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="INGEME" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -2152,7 +2152,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -3426,7 +3426,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3999,7 +3999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4851,22 +4851,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>-152</t>
+          <t>5589</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11/1/2024</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FERNANDEZ DE ENCISO /ALT/ 3610</t>
+          <t>ARCOS 1520</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4881,12 +4881,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>798984311</t>
+          <t>799540526</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>El poste esta pegado al arbol ver la foto adjunta</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -4896,26 +4896,26 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>-58.513363</v>
+        <v>-58.449125</v>
       </c>
       <c r="N11" t="n">
-        <v>-34.605473</v>
+        <v>-34.565958</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4925,29 +4925,29 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>DEV-F</t>
+          <t>BLO-M</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.1DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5589</t>
+          <t>5884</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>11/7/2024</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ARCOS 1520</t>
+          <t>OLLEROS 2952</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4967,12 +4967,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>799540526</t>
+          <t>799450967</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Terminar transferencia, retirar columna vieja</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -4994,24 +4994,24 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>-58.449125</v>
+        <v>-58.447022</v>
       </c>
       <c r="N12" t="n">
-        <v>-34.565958</v>
+        <v>-34.575873</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>BLO-M</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -5023,22 +5023,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5884</t>
+          <t>4579</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11/7/2024</t>
+          <t>1/9/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>OLLEROS 2952</t>
+          <t>PASCO 10</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -5053,12 +5053,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>799450967</t>
+          <t>802438793</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Terminar transferencia, retirar columna vieja</t>
+          <t>PIcada</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -5073,21 +5073,21 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>-58.447022</v>
+        <v>-58.397512</v>
       </c>
       <c r="N13" t="n">
-        <v>-34.575873</v>
+        <v>-34.609923</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -5097,7 +5097,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -5109,22 +5109,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>4528</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12/21/2024</t>
+          <t>1/16/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MERCEDES 254</t>
+          <t>BARCO CENTENERA DEL 545</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -5139,12 +5139,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>802774521</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Colocar R200 para pedir traspaso de equipo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -5166,51 +5166,51 @@
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>-58.484232</v>
+        <v>-58.440625</v>
       </c>
       <c r="N14" t="n">
-        <v>-34.631431</v>
+        <v>-34.625499</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>PCH-C</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4579</t>
+          <t>4862</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1/9/2025</t>
+          <t>1/23/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PASCO 10</t>
+          <t>ARCOS 2263</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5225,12 +5225,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>802438793</t>
+          <t>802857379</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>PIcada</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -5245,31 +5245,31 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>-58.397512</v>
+        <v>-58.455082</v>
       </c>
       <c r="N15" t="n">
-        <v>-34.609923</v>
+        <v>-34.558883</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>BLO-P</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -5281,22 +5281,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4528</t>
+          <t>4696</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1/16/2025</t>
+          <t>2/10/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BARCO CENTENERA DEL 545</t>
+          <t>YERBAL 489</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5311,12 +5311,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>802774521</t>
+          <t>803607520</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Desmonte de columna ya traspasaron nodo</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -5326,7 +5326,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -5338,10 +5338,10 @@
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>-58.440625</v>
+        <v>-58.438053</v>
       </c>
       <c r="N16" t="n">
-        <v>-34.625499</v>
+        <v>-34.617481</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -5355,7 +5355,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>PCH-C</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -5367,22 +5367,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4680</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1/22/2025</t>
+          <t>2/14/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CUENCA 3345</t>
+          <t>CHACO 195</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5397,12 +5397,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>803607699</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Desmontar columna personal propio traspaso nodo</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -5424,24 +5424,24 @@
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.496935</v>
+        <v>-58.431522</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.599084</v>
+        <v>-34.617523</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -5453,22 +5453,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4862</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1/23/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ARCOS 2263</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5483,12 +5483,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>802857379</t>
+          <t>804309655</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -5507,27 +5507,27 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.455082</v>
+        <v>-58.441405</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.558883</v>
+        <v>-34.594348</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>BLO-P</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -5539,22 +5539,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4696</t>
+          <t>5657</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2/10/2025</t>
+          <t>4/23/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>YERBAL 489</t>
+          <t>COCHABAMBA 2207</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5569,12 +5569,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>803607520</t>
+          <t>804903806</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Desmonte de columna ya traspasaron nodo</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -5584,7 +5584,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -5593,17 +5593,17 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.438053</v>
+        <v>-58.396135</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.617481</v>
+        <v>-34.624285</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -5613,7 +5613,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -5625,22 +5625,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>5682</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2/14/2025</t>
+          <t>4/29/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CHACO 195</t>
+          <t>República Bolivariana de Venezuela 2701</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5655,12 +5655,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>803607699</t>
+          <t>805507294</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Desmontar columna personal propio traspaso nodo</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -5675,21 +5675,21 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L20" t="n">
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.431522</v>
+        <v>-58.404913</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.617523</v>
+        <v>-34.615857</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -5699,7 +5699,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -5711,22 +5711,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>5708</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3/13/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TANDIL 4746</t>
+          <t>SARMIENTO 1741</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5741,10 +5741,14 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>803983204</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>805579089</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Pendiente de traspaso nodo y fuente</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -5752,36 +5756,36 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.487666</v>
+        <v>-58.391419</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.649704</v>
+        <v>-34.605543</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PAV-N</t>
+          <t>CEN-E</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -5793,22 +5797,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>5731</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>RIOBAMBA 659</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5823,12 +5827,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>805579188</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -5850,14 +5854,14 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.441405</v>
+        <v>-58.394118</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.594348</v>
+        <v>-34.601416</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -5867,7 +5871,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>RET-H</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -5879,22 +5883,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5909,10 +5913,14 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>804309801</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>805791908</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -5932,24 +5940,24 @@
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.483821</v>
+        <v>-58.451835</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.677698</v>
+        <v>-34.562646</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -5961,22 +5969,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5657</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4/23/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COCHABAMBA 2207</t>
+          <t>MAZA 181</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5991,12 +5999,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>807215439</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -6006,7 +6014,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -6015,17 +6023,17 @@
         </is>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.396135</v>
+        <v>-58.416477</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.624285</v>
+        <v>-34.61303</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -6035,7 +6043,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>CLI-I</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -6047,17 +6055,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5682</t>
+          <t>6076</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>República Bolivariana de Venezuela 2701</t>
+          <t>MATHEU 727</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -6077,14 +6085,10 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>805507294</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Picada</t>
-        </is>
-      </c>
+          <t>ICD31456940</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -6092,22 +6096,22 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L25" t="n">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.404913</v>
+        <v>-58.400169</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.615857</v>
+        <v>-34.617784</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
@@ -6121,7 +6125,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CEN-N</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -6133,22 +6137,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>6284</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>6/30/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>CHILE 2561</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -6163,14 +6167,10 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>805579089</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
-        </is>
-      </c>
+          <t>807851584</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -6178,7 +6178,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -6190,14 +6190,14 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.391419</v>
+        <v>-58.401827</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.605543</v>
+        <v>-34.617667</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CEN-E</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -6219,22 +6219,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5731</t>
+          <t>5999</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>8/12/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RIOBAMBA 659</t>
+          <t>MARMOL, JOSE 228</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -6249,12 +6249,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>808918687</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -6264,7 +6264,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -6273,13 +6273,13 @@
         </is>
       </c>
       <c r="L27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.394118</v>
+        <v>-58.425858</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.601416</v>
+        <v>-34.61629</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -6293,7 +6293,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -6305,22 +6305,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -6335,12 +6335,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>ICD30508311</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -6350,36 +6350,36 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L28" t="n">
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.451835</v>
+        <v>-58.435017</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.562646</v>
+        <v>-34.622044</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -6391,22 +6391,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MAZA 181</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6421,12 +6421,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>807215439</t>
+          <t>ICD30593982</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -6441,21 +6441,21 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L29" t="n">
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.416477</v>
+        <v>-58.443232</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.61303</v>
+        <v>-34.620007</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
@@ -6465,7 +6465,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>CLI-I</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -6477,22 +6477,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6076</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MATHEU 727</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -6507,10 +6507,14 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>809910087</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Picada</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -6518,7 +6522,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Nodo TLC</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -6530,14 +6534,14 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.400169</v>
+        <v>-58.442045</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.617784</v>
+        <v>-34.594303</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -6547,7 +6551,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>CEN-N</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -6559,22 +6563,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6284</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>6/30/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CHILE 2561</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -6589,10 +6593,14 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>807851584</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Picada</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -6609,27 +6617,27 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.401827</v>
+        <v>-58.444996</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.617667</v>
+        <v>-34.564443</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -6641,22 +6649,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -6671,12 +6679,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -6686,7 +6694,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -6698,14 +6706,14 @@
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.425858</v>
+        <v>-58.4018</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.61629</v>
+        <v>-34.590471</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -6715,7 +6723,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -6727,22 +6735,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -6757,12 +6765,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -6784,14 +6792,14 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.435017</v>
+        <v>-58.436262</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.622044</v>
+        <v>-34.600478</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -6801,7 +6809,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -6813,22 +6821,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>LAMBARE 864</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -6843,12 +6851,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>811453866</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -6858,26 +6866,26 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.443232</v>
+        <v>-58.430579</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.620007</v>
+        <v>-34.604908</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -6887,7 +6895,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>ALM-M</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -6899,22 +6907,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>3875</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>Castelli 60</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -6929,41 +6937,29 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Picada</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+          <t>traspaso propio tlc coloco columna</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.442045</v>
+        <v>-58.404691</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.594303</v>
+        <v>-34.609194</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -6973,514 +6969,10 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>-649</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>10/23/2025</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Arribeños 1438</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Picada</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L36" t="n">
-        <v>0</v>
-      </c>
-      <c r="M36" t="n">
-        <v>-58.444996</v>
-      </c>
-      <c r="N36" t="n">
-        <v>-34.564443</v>
-      </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="P36" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q36" t="inlineStr">
-        <is>
-          <t>BLO-K</t>
-        </is>
-      </c>
-      <c r="R36" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>5749</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>10/27/2025</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>01230434</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
-      </c>
-      <c r="M37" t="n">
-        <v>-58.4018</v>
-      </c>
-      <c r="N37" t="n">
-        <v>-34.590471</v>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>Recoleta</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>AGU-F</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>S01150217</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>10/29/2025</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Vera 311</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>01230602</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Traspasar Fuente</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>Fuente Teco</t>
-        </is>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="L38" t="n">
-        <v>1</v>
-      </c>
-      <c r="M38" t="n">
-        <v>-58.436262</v>
-      </c>
-      <c r="N38" t="n">
-        <v>-34.600478</v>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q38" t="inlineStr">
-        <is>
-          <t>CLI-O</t>
-        </is>
-      </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>-670</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>11/10/2025</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Timoteo Gordillo 1666</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>810651269</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L39" t="n">
-        <v>1</v>
-      </c>
-      <c r="M39" t="n">
-        <v>-58.510994</v>
-      </c>
-      <c r="N39" t="n">
-        <v>-34.655027</v>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>PAV-J</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>8043</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>1/8/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>LAMBARE 864</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>811453866</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>corroida</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L40" t="n">
-        <v>1</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-58.430579</v>
-      </c>
-      <c r="N40" t="n">
-        <v>-34.604908</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>ALM-M</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>3875</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>1/16/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Castelli 60</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>traspaso propio tlc coloco columna</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="n">
-        <v>1</v>
-      </c>
-      <c r="M41" t="n">
-        <v>-58.404691</v>
-      </c>
-      <c r="N41" t="n">
-        <v>-34.609194</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>CLI-D</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -7497,7 +6989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7595,84 +7087,592 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>-152</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>11/1/2024</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>FERNANDEZ DE ENCISO /ALT/ 3610</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>798984311</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>El poste esta pegado al arbol ver la foto adjunta</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>-58.513363</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-34.605473</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>DEV-F</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.1DEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>4082</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>12/21/2024</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MERCEDES 254</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>801901755</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Colocar R200 para pedir traspaso de equipo</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>-58.484232</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-34.631431</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>DEV-L</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ARATO-25058.PO.2DEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4680</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1/22/2025</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CUENCA 3345</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>802843289</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Picada</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>-58.496935</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-34.599084</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>PUE-B</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>6029</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3/13/2025</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TANDIL 4746</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>803983204</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-58.487666</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-34.649704</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>PAV-N</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4179</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3/27/2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ZELARRAYAN 6147</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>804309801</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-58.483821</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-34.677698</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>PAV-Q</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>7570</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>10/6/2025</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>Pendiente ADM</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Colocar R150 o R200</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>Nodo Teco</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Pasante</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="L7" t="n">
         <v>1</v>
       </c>
-      <c r="M2" t="n">
+      <c r="M7" t="n">
         <v>-58.465176</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N7" t="n">
         <v>-34.680979</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Boedo</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>PAV-U</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>-670</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11/10/2025</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Timoteo Gordillo 1666</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>810651269</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-58.510994</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-34.655027</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>PAV-J</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-20 09:50:01)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1267,22 +1267,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>-152</t>
+          <t>5589</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>11/1/2024</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>FERNANDEZ DE ENCISO /ALT/ 3610</t>
+          <t>ARCOS 1520</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1292,17 +1292,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Propio</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>798984311</t>
+          <t>799540526</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>El poste esta pegado al arbol ver la foto adjunta</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1312,26 +1312,26 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>-58.513363</v>
+        <v>-58.449125</v>
       </c>
       <c r="N11" t="n">
-        <v>-34.605473</v>
+        <v>-34.565958</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1341,29 +1341,29 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>DEV-F</t>
+          <t>BLO-M</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.1DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5589</t>
+          <t>5884</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>11/7/2024</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ARCOS 1520</t>
+          <t>OLLEROS 2952</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>799540526</t>
+          <t>799450967</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Terminar transferencia, retirar columna vieja</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1410,24 +1410,24 @@
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>-58.449125</v>
+        <v>-58.447022</v>
       </c>
       <c r="N12" t="n">
-        <v>-34.565958</v>
+        <v>-34.575873</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>BLO-M</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1439,22 +1439,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>5884</t>
+          <t>4082</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>11/7/2024</t>
+          <t>12/21/2024</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>OLLEROS 2952</t>
+          <t>MERCEDES 254</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1464,17 +1464,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>799450967</t>
+          <t>801901755</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Terminar transferencia, retirar columna vieja</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1493,54 +1493,54 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>-58.447022</v>
+        <v>-58.484232</v>
       </c>
       <c r="N13" t="n">
-        <v>-34.575873</v>
+        <v>-34.631431</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>4579</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>12/21/2024</t>
+          <t>1/9/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MERCEDES 254</t>
+          <t>PASCO 10</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1550,17 +1550,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Propio</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>802438793</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Colocar R200 para pedir traspaso de equipo</t>
+          <t>PIcada</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1575,58 +1575,58 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>-58.484232</v>
+        <v>-58.397512</v>
       </c>
       <c r="N14" t="n">
-        <v>-34.631431</v>
+        <v>-34.609923</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4579</t>
+          <t>4528</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1/9/2025</t>
+          <t>1/16/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PASCO 10</t>
+          <t>BARCO CENTENERA DEL 545</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1641,12 +1641,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>802438793</t>
+          <t>802774521</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>PIcada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1656,26 +1656,26 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L15" t="n">
         <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>-58.397512</v>
+        <v>-58.440625</v>
       </c>
       <c r="N15" t="n">
-        <v>-34.609923</v>
+        <v>-34.625499</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1685,7 +1685,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>PCH-C</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1697,22 +1697,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4528</t>
+          <t>4680</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1/16/2025</t>
+          <t>1/22/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BARCO CENTENERA DEL 545</t>
+          <t>CUENCA 3345</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1722,17 +1722,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>802774521</t>
+          <t>802843289</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1754,24 +1754,24 @@
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>-58.440625</v>
+        <v>-58.496935</v>
       </c>
       <c r="N16" t="n">
-        <v>-34.625499</v>
+        <v>-34.599084</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>PCH-C</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1783,22 +1783,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4680</t>
+          <t>4862</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1/22/2025</t>
+          <t>1/23/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CUENCA 3345</t>
+          <t>ARCOS 2263</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1808,17 +1808,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Propio</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>802857379</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1837,17 +1837,17 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.496935</v>
+        <v>-58.455082</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.599084</v>
+        <v>-34.558883</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>BLO-P</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1869,22 +1869,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4862</t>
+          <t>4696</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>1/23/2025</t>
+          <t>2/10/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ARCOS 2263</t>
+          <t>YERBAL 489</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1899,12 +1899,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>802857379</t>
+          <t>803607520</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Desmonte de columna ya traspasaron nodo</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1923,27 +1923,27 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.455082</v>
+        <v>-58.438053</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.558883</v>
+        <v>-34.617481</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>BLO-P</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1955,17 +1955,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4696</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2/10/2025</t>
+          <t>2/14/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>YERBAL 489</t>
+          <t>CHACO 195</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>803607520</t>
+          <t>803607699</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Desmonte de columna ya traspasaron nodo</t>
+          <t>Desmontar columna personal propio traspaso nodo</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2012,10 +2012,10 @@
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.438053</v>
+        <v>-58.431522</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.617481</v>
+        <v>-34.617523</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2041,22 +2041,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2/14/2025</t>
+          <t>3/13/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CHACO 195</t>
+          <t>TANDIL 4746</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2066,17 +2066,17 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>803607699</t>
+          <t>803983204</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Desmontar columna personal propio traspaso nodo</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2086,36 +2086,36 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.431522</v>
+        <v>-58.487666</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.617523</v>
+        <v>-34.649704</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>PAV-N</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2127,22 +2127,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3/13/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TANDIL 4746</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2152,15 +2152,19 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Propio</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>803983204</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr"/>
+          <t>804309655</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2168,36 +2172,36 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.487666</v>
+        <v>-58.441405</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.649704</v>
+        <v>-34.594348</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PAV-N</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2209,7 +2213,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2219,12 +2223,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2234,17 +2238,17 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>804309801</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2266,14 +2270,14 @@
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.441405</v>
+        <v>-58.483821</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.594348</v>
+        <v>-34.677698</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2283,7 +2287,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2295,22 +2299,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>5657</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>4/23/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>COCHABAMBA 2207</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2320,15 +2324,19 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Propio</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>804309801</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>804903806</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>picada</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2336,7 +2344,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2345,17 +2353,17 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.483821</v>
+        <v>-58.396135</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.677698</v>
+        <v>-34.624285</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2365,7 +2373,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2377,17 +2385,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5657</t>
+          <t>5682</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4/23/2025</t>
+          <t>4/29/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COCHABAMBA 2207</t>
+          <t>República Bolivariana de Venezuela 2701</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2407,12 +2415,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>805507294</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2422,26 +2430,26 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.396135</v>
+        <v>-58.404913</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.624285</v>
+        <v>-34.615857</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2451,7 +2459,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2463,22 +2471,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5682</t>
+          <t>5708</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>República Bolivariana de Venezuela 2701</t>
+          <t>SARMIENTO 1741</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2493,12 +2501,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>805507294</t>
+          <t>805579089</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Pendiente de traspaso nodo y fuente</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2508,26 +2516,26 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L25" t="n">
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.404913</v>
+        <v>-58.391419</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.615857</v>
+        <v>-34.605543</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2537,7 +2545,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CEN-E</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2549,7 +2557,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>5731</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2559,12 +2567,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>RIOBAMBA 659</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2579,12 +2587,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>805579089</t>
+          <t>805579188</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
+          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2594,7 +2602,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2606,14 +2614,14 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.391419</v>
+        <v>-58.394118</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.605543</v>
+        <v>-34.601416</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
@@ -2623,7 +2631,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CEN-E</t>
+          <t>RET-H</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2635,22 +2643,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5731</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>RIOBAMBA 659</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2665,12 +2673,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2692,24 +2700,24 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.394118</v>
+        <v>-58.451835</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.601416</v>
+        <v>-34.562646</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2721,22 +2729,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>MAZA 181</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2751,12 +2759,12 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>807215439</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -2778,24 +2786,24 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.451835</v>
+        <v>-58.416477</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.562646</v>
+        <v>-34.61303</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>CLI-I</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2807,22 +2815,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>6076</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MAZA 181</t>
+          <t>MATHEU 727</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2837,14 +2845,10 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>807215439</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Picada</t>
-        </is>
-      </c>
+          <t>ICD31456940</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2852,7 +2856,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2864,10 +2868,10 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.416477</v>
+        <v>-58.400169</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.61303</v>
+        <v>-34.617784</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2881,7 +2885,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>CLI-I</t>
+          <t>CEN-N</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2893,17 +2897,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6076</t>
+          <t>6284</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>6/30/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MATHEU 727</t>
+          <t>CHILE 2561</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2923,7 +2927,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
+          <t>807851584</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -2934,7 +2938,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Nodo TLC</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2946,10 +2950,10 @@
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.400169</v>
+        <v>-58.401827</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.617784</v>
+        <v>-34.617667</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2963,7 +2967,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>CEN-N</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2975,22 +2979,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6284</t>
+          <t>5999</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>6/30/2025</t>
+          <t>8/12/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CHILE 2561</t>
+          <t>MARMOL, JOSE 228</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3005,10 +3009,14 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>807851584</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr"/>
+          <t>808918687</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -3016,7 +3024,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3025,13 +3033,13 @@
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.401827</v>
+        <v>-58.425858</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.617667</v>
+        <v>-34.61629</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3045,7 +3053,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3057,22 +3065,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3087,12 +3095,12 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>ICD30508311</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3107,21 +3115,21 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.425858</v>
+        <v>-58.435017</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.61629</v>
+        <v>-34.622044</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3131,7 +3139,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3143,17 +3151,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -3173,12 +3181,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>ICD30593982</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3188,7 +3196,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3200,10 +3208,10 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.435017</v>
+        <v>-58.443232</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.622044</v>
+        <v>-34.620007</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3217,7 +3225,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3229,22 +3237,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3259,12 +3267,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>809910087</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3279,21 +3287,21 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L34" t="n">
         <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.443232</v>
+        <v>-58.442045</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.620007</v>
+        <v>-34.594303</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
@@ -3303,7 +3311,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3315,22 +3323,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>7570</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>10/6/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3340,17 +3348,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3372,14 +3380,14 @@
         <v>1</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.442045</v>
+        <v>-58.465176</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.594303</v>
+        <v>-34.680979</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3389,7 +3397,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3401,22 +3409,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3426,7 +3434,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Propio</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3436,7 +3444,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Colocar R150 o R200</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3455,27 +3463,27 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.465176</v>
+        <v>-58.444996</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.680979</v>
+        <v>-34.564443</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3487,22 +3495,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>-649</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10/23/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Arribeños 1438</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3517,12 +3525,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3544,24 +3552,24 @@
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.444996</v>
+        <v>-58.4018</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.564443</v>
+        <v>-34.590471</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>BLO-K</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3573,22 +3581,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5749</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3603,12 +3611,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3618,26 +3626,26 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.4018</v>
+        <v>-58.436262</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.590471</v>
+        <v>-34.600478</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3647,7 +3655,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3659,22 +3667,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S01150217</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Vera 311</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3684,17 +3692,17 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Propio</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>01230602</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Traspasar Fuente</t>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3704,36 +3712,36 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.436262</v>
+        <v>-58.510994</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.600478</v>
+        <v>-34.655027</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3745,22 +3753,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>LAMBARE 864</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3770,17 +3778,17 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Propio</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>811453866</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3802,24 +3810,24 @@
         <v>1</v>
       </c>
       <c r="M40" t="n">
-        <v>-58.510994</v>
+        <v>-58.430579</v>
       </c>
       <c r="N40" t="n">
-        <v>-34.655027</v>
+        <v>-34.604908</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>ALM-M</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
@@ -3831,22 +3839,22 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>8043</t>
+          <t>3875</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LAMBARE 864</t>
+          <t>Castelli 60</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3861,37 +3869,25 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>811453866</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>corroida</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+          <t>traspaso propio tlc coloco columna</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
       <c r="L41" t="n">
         <v>1</v>
       </c>
       <c r="M41" t="n">
-        <v>-58.430579</v>
+        <v>-58.404691</v>
       </c>
       <c r="N41" t="n">
-        <v>-34.604908</v>
+        <v>-34.609194</v>
       </c>
       <c r="O41" t="inlineStr">
         <is>
@@ -3905,84 +3901,10 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>ALM-M</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>3875</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>1/16/2026</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Castelli 60</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Propio</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>traspaso propio tlc coloco columna</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr"/>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
-      <c r="L42" t="n">
-        <v>1</v>
-      </c>
-      <c r="M42" t="n">
-        <v>-58.404691</v>
-      </c>
-      <c r="N42" t="n">
-        <v>-34.609194</v>
-      </c>
-      <c r="O42" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>CLI-D</t>
-        </is>
-      </c>
-      <c r="R42" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -6989,7 +6911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7087,22 +7009,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>-152</t>
+          <t>4082</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11/1/2024</t>
+          <t>12/21/2024</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FERNANDEZ DE ENCISO /ALT/ 3610</t>
+          <t>MERCEDES 254</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -7117,12 +7039,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>798984311</t>
+          <t>801901755</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>El poste esta pegado al arbol ver la foto adjunta</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7132,22 +7054,22 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Poste</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>-58.513363</v>
+        <v>-58.484232</v>
       </c>
       <c r="N2" t="n">
-        <v>-34.605473</v>
+        <v>-34.631431</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -7161,34 +7083,34 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DEV-F</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.1DEV</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>4680</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12/21/2024</t>
+          <t>1/22/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>MERCEDES 254</t>
+          <t>CUENCA 3345</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -7203,12 +7125,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>802843289</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Colocar R200 para pedir traspaso de equipo</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7230,14 +7152,14 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>-58.484232</v>
+        <v>-58.496935</v>
       </c>
       <c r="N3" t="n">
-        <v>-34.631431</v>
+        <v>-34.599084</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -7247,34 +7169,34 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4680</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1/22/2025</t>
+          <t>3/13/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CUENCA 3345</t>
+          <t>TANDIL 4746</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -7289,12 +7211,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>803983204</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7304,26 +7226,26 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-58.496935</v>
+        <v>-58.487666</v>
       </c>
       <c r="N4" t="n">
-        <v>-34.599084</v>
+        <v>-34.649704</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
@@ -7333,7 +7255,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>PAV-N</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -7345,22 +7267,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3/13/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TANDIL 4746</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7375,10 +7297,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>803983204</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>804309801</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -7386,36 +7312,36 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>-58.487666</v>
+        <v>-58.483821</v>
       </c>
       <c r="N5" t="n">
-        <v>-34.649704</v>
+        <v>-34.677698</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PAV-N</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -7427,17 +7353,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>7570</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>10/6/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -7457,10 +7383,14 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>804309801</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr"/>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -7480,10 +7410,10 @@
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>-58.483821</v>
+        <v>-58.465176</v>
       </c>
       <c r="N6" t="n">
-        <v>-34.677698</v>
+        <v>-34.680979</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -7497,7 +7427,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -7509,22 +7439,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -7539,12 +7469,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Colocar R150 o R200</t>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -7554,7 +7484,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -7566,113 +7496,27 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>-58.465176</v>
+        <v>-58.510994</v>
       </c>
       <c r="N7" t="n">
-        <v>-34.680979</v>
+        <v>-34.655027</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>-670</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>11/10/2025</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Timoteo Gordillo 1666</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>810651269</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Cambiar columna de lugar la actual es un poste ex Cablevision correrla ya que el vecino reclama obstruccion de la cochera</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" t="n">
-        <v>-58.510994</v>
-      </c>
-      <c r="N8" t="n">
-        <v>-34.655027</v>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>PAV-J</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-05-27 07:23:10)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -2242,7 +2242,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -6697,7 +6697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7053,22 +7053,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7083,12 +7083,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>804309801</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -7110,199 +7110,27 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>-58.483821</v>
+        <v>-58.510994</v>
       </c>
       <c r="N5" t="n">
-        <v>-34.677698</v>
+        <v>-34.655027</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>7570</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>10/6/2025</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="n">
-        <v>-58.465176</v>
-      </c>
-      <c r="N6" t="n">
-        <v>-34.680979</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>PAV-U</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>-670</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>11/10/2025</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Timoteo Gordillo 1666</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>810651269</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M7" t="n">
-        <v>-58.510994</v>
-      </c>
-      <c r="N7" t="n">
-        <v>-34.655027</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Devoto</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>PAV-J</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -7319,7 +7147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7589,22 +7417,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -7619,12 +7447,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>804309801</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7634,22 +7462,22 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L4" t="n">
         <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>-58.435017</v>
+        <v>-58.483821</v>
       </c>
       <c r="N4" t="n">
-        <v>-34.622044</v>
+        <v>-34.677698</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -7663,7 +7491,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -7675,17 +7503,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -7705,12 +7533,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>ICD30508311</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -7720,7 +7548,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -7732,27 +7560,199 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
+        <v>-58.435017</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-34.622044</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>PCH-M</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4698</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8/29/2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>REPETTO, NICOLAS, DR. 93</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ICD30593982</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
         <v>-58.443232</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N6" t="n">
         <v>-34.620007</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Boedo</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>PCH-G</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>7570</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/6/2025</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-58.465176</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-34.680979</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-02 15:37:39)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -445,17 +445,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -537,17 +537,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>ICD30334341</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>ICD30334341</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -619,17 +619,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>791764767</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>791764767</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -705,17 +705,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>791898287</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>791898287</t>
         </is>
       </c>
       <c r="H4" t="inlineStr"/>
@@ -787,17 +787,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>798385574</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>798385574</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -873,17 +873,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>798513095</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>798513095</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -955,17 +955,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>798897149</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>798897149</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1037,17 +1037,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>798307407</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>798307407</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1123,17 +1123,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>780340125</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>780340125</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1209,17 +1209,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>797752816</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>797752816</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1291,17 +1291,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>799540526</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>799540526</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1377,17 +1377,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>799450967</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>799450967</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1463,17 +1463,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>801901755</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>801901755</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1549,17 +1549,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>802438793</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>802438793</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1635,17 +1635,17 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>802774521</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>802774521</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>802843289</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>802843289</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1807,17 +1807,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>802857379</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>802857379</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1893,17 +1893,17 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>803607520</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>803607520</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1979,17 +1979,17 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>803607699</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>803607699</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2065,17 +2065,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>803983204</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>803983204</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2151,17 +2151,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>804309655</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>804309655</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2237,17 +2237,17 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>804309801</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>804309801</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2323,17 +2323,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>804903806</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>804903806</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2409,17 +2409,17 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>805507294</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>805507294</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2495,17 +2495,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>805579089</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>ROWING</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>805579089</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2581,17 +2581,17 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>805579188</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>805579188</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2667,17 +2667,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>805791908</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>805791908</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2753,17 +2753,17 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>807215439</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>807215439</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2839,17 +2839,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>ICD31456940</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>ICD31456940</t>
         </is>
       </c>
       <c r="H29" t="inlineStr"/>
@@ -2921,17 +2921,17 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>807851584</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>807851584</t>
         </is>
       </c>
       <c r="H30" t="inlineStr"/>
@@ -3003,17 +3003,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
+          <t>808918687</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>808918687</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3089,17 +3089,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t>ICD30508311</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>ICD30508311</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3175,17 +3175,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
+          <t>ICD30593982</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>ICD30593982</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3261,17 +3261,17 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
+          <t>809910087</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>809910087</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3347,17 +3347,17 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3433,17 +3433,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3519,17 +3519,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
+          <t>01230434</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>01230434</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3605,17 +3605,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
+          <t>01230602</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>01230602</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3691,17 +3691,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>810651269</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>810651269</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3777,17 +3777,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>811453866</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>811453866</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3863,17 +3863,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3951,17 +3951,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -4043,17 +4043,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>ICD30334341</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>ICD30334341</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -4125,17 +4125,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>791764767</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>791764767</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -4211,17 +4211,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>798897149</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>798897149</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -4293,17 +4293,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>01230434</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>PEBCOM</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>01230434</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -4393,17 +4393,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -4485,17 +4485,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>791898287</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>791898287</t>
         </is>
       </c>
       <c r="H2" t="inlineStr"/>
@@ -4567,17 +4567,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>798307407</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>798307407</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -4653,17 +4653,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>780340125</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>780340125</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -4739,17 +4739,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>797752816</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>797752816</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -4821,17 +4821,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>799540526</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>799540526</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -4907,17 +4907,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>799450967</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>799450967</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -4993,17 +4993,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>802857379</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>802857379</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -5079,17 +5079,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>804309655</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>804309655</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -5165,17 +5165,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>805791908</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>805791908</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -5251,17 +5251,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>809910087</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>809910087</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -5337,17 +5337,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -5423,17 +5423,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>01230602</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>NEW</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>01230602</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -5523,17 +5523,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -5615,17 +5615,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>798385574</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>798385574</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -5701,17 +5701,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>798513095</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>798513095</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -5783,17 +5783,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>802438793</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>802438793</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -5869,17 +5869,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>802774521</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>802774521</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -5955,17 +5955,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>804903806</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>804903806</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -6041,17 +6041,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>805507294</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>805507294</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -6127,17 +6127,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>805579188</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>805579188</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -6213,17 +6213,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>807215439</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>807215439</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -6299,17 +6299,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>ICD31456940</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>ICD31456940</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -6381,17 +6381,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>807851584</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>807851584</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -6463,17 +6463,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>808918687</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>808918687</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -6549,17 +6549,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>811453866</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>811453866</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -6635,17 +6635,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -6723,17 +6723,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -6815,17 +6815,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>801901755</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>801901755</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -6901,17 +6901,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>802843289</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>802843289</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -6987,17 +6987,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>803983204</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>803983204</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -7073,17 +7073,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>810651269</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>INGEME</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>810651269</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -7173,17 +7173,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -7265,17 +7265,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>803607520</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>803607520</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -7351,17 +7351,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>803607699</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>803607699</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -7437,17 +7437,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>804309801</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>804309801</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -7523,17 +7523,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>ICD30508311</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>ICD30508311</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -7609,17 +7609,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>ICD30593982</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>ICD30593982</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -7695,17 +7695,17 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -7795,17 +7795,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Proveedor Asignado</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>OT</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -7887,17 +7887,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>805579089</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Pendiente de Traspaso PROPIO</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>ROWING</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>805579089</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-05 17:13:27)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1103,17 +1103,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>7758</t>
+          <t>5589</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2/20/2024</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ZABALA 2844</t>
+          <t>ARCOS 1520</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>780340125</t>
+          <t>799540526</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>cambiar columna y emprolijar cables y cajas de empalme que se ven en las fotos</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1157,13 +1157,13 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>-58.452328</v>
+        <v>-58.449125</v>
       </c>
       <c r="N9" t="n">
-        <v>-34.572196</v>
+        <v>-34.565958</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>ATH-Q</t>
+          <t>BLO-M</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1189,17 +1189,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>-143</t>
+          <t>5884</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10/7/2024</t>
+          <t>11/7/2024</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ /ALT/ 2261</t>
+          <t>OLLEROS 2952</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>797752816</t>
+          <t>799450967</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1222,7 +1222,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Terminar transferencia, retirar columna vieja</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -1242,24 +1246,24 @@
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>-58.458864</v>
+        <v>-58.447022</v>
       </c>
       <c r="N10" t="n">
-        <v>-34.561167</v>
+        <v>-34.575873</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>COG-H</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1271,22 +1275,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>5589</t>
+          <t>4082</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/21/2024</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ARCOS 1520</t>
+          <t>MERCEDES 254</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1296,17 +1300,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>799540526</t>
+          <t>801901755</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1325,17 +1329,17 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>-58.449125</v>
+        <v>-58.484232</v>
       </c>
       <c r="N11" t="n">
-        <v>-34.565958</v>
+        <v>-34.631431</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1345,34 +1349,34 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>BLO-M</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>5884</t>
+          <t>4579</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>11/7/2024</t>
+          <t>1/9/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OLLEROS 2952</t>
+          <t>PASCO 10</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1382,17 +1386,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>799450967</t>
+          <t>802438793</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Terminar transferencia, retirar columna vieja</t>
+          <t>PIcada</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1407,21 +1411,21 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>-58.447022</v>
+        <v>-58.397512</v>
       </c>
       <c r="N12" t="n">
-        <v>-34.575873</v>
+        <v>-34.609923</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1431,7 +1435,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
@@ -1443,22 +1447,22 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>4528</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>12/21/2024</t>
+          <t>1/16/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MERCEDES 254</t>
+          <t>BARCO CENTENERA DEL 545</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1468,17 +1472,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>802774521</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1488,7 +1492,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1500,51 +1504,51 @@
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>-58.484232</v>
+        <v>-58.440625</v>
       </c>
       <c r="N13" t="n">
-        <v>-34.631431</v>
+        <v>-34.625499</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>PCH-C</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4579</t>
+          <t>4680</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1/9/2025</t>
+          <t>1/22/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>PASCO 10</t>
+          <t>CUENCA 3345</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1554,17 +1558,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>802438793</t>
+          <t>802843289</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>PIcada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1579,31 +1583,31 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L14" t="n">
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>-58.397512</v>
+        <v>-58.496935</v>
       </c>
       <c r="N14" t="n">
-        <v>-34.609923</v>
+        <v>-34.599084</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1615,22 +1619,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4528</t>
+          <t>4862</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1/16/2025</t>
+          <t>1/23/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BARCO CENTENERA DEL 545</t>
+          <t>ARCOS 2263</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1640,17 +1644,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>802774521</t>
+          <t>802857379</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1660,7 +1664,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -1669,27 +1673,27 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>-58.440625</v>
+        <v>-58.455082</v>
       </c>
       <c r="N15" t="n">
-        <v>-34.625499</v>
+        <v>-34.558883</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>PCH-C</t>
+          <t>BLO-P</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1701,22 +1705,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4680</t>
+          <t>4696</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>1/22/2025</t>
+          <t>2/10/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CUENCA 3345</t>
+          <t>YERBAL 489</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1726,17 +1730,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>803607520</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Desmonte de columna ya traspasaron nodo</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1758,24 +1762,24 @@
         <v>1</v>
       </c>
       <c r="M16" t="n">
-        <v>-58.496935</v>
+        <v>-58.438053</v>
       </c>
       <c r="N16" t="n">
-        <v>-34.599084</v>
+        <v>-34.617481</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1787,22 +1791,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4862</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>1/23/2025</t>
+          <t>2/14/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ARCOS 2263</t>
+          <t>CHACO 195</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1812,17 +1816,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>802857379</t>
+          <t>803607699</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Desmontar columna personal propio traspaso nodo</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1841,27 +1845,27 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.455082</v>
+        <v>-58.431522</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.558883</v>
+        <v>-34.617523</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>BLO-P</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1873,22 +1877,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4696</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2/10/2025</t>
+          <t>3/13/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>YERBAL 489</t>
+          <t>TANDIL 4746</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1898,17 +1902,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>803607520</t>
+          <t>803983204</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Desmonte de columna ya traspasaron nodo</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1918,36 +1922,36 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.438053</v>
+        <v>-58.487666</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.617481</v>
+        <v>-34.649704</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>PAV-N</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1959,22 +1963,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2/14/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>CHACO 195</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1984,17 +1988,17 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>803607699</t>
+          <t>804309655</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Desmontar columna personal propio traspaso nodo</t>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2016,14 +2020,14 @@
         <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.431522</v>
+        <v>-58.441405</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.617523</v>
+        <v>-34.594348</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -2033,7 +2037,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2045,22 +2049,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3/13/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TANDIL 4746</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2070,12 +2074,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>803983204</t>
+          <t>804309801</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2090,36 +2094,36 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.487666</v>
+        <v>-58.483821</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.649704</v>
+        <v>-34.677698</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PAV-N</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2131,22 +2135,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>5657</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>4/23/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>COCHABAMBA 2207</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2156,17 +2160,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>804903806</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2176,7 +2180,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2185,17 +2189,17 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.441405</v>
+        <v>-58.396135</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.594348</v>
+        <v>-34.624285</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2205,7 +2209,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2217,22 +2221,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>5682</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>4/29/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>República Bolivariana de Venezuela 2701</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2242,17 +2246,17 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>804309801</t>
+          <t>805507294</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2267,21 +2271,21 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L22" t="n">
         <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.483821</v>
+        <v>-58.404913</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.677698</v>
+        <v>-34.615857</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2291,7 +2295,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2303,22 +2307,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5657</t>
+          <t>5708</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4/23/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COCHABAMBA 2207</t>
+          <t>SARMIENTO 1741</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2328,17 +2332,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>805579089</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>ROWING</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Pendiente de traspaso nodo y fuente</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2348,7 +2352,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2357,13 +2361,13 @@
         </is>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.396135</v>
+        <v>-58.391419</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.624285</v>
+        <v>-34.605543</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
@@ -2377,7 +2381,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>CEN-E</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2389,17 +2393,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5682</t>
+          <t>5731</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>República Bolivariana de Venezuela 2701</t>
+          <t>RIOBAMBA 659</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2414,7 +2418,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>805507294</t>
+          <t>805579188</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -2424,7 +2428,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2439,17 +2443,17 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L24" t="n">
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.404913</v>
+        <v>-58.394118</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.615857</v>
+        <v>-34.601416</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
@@ -2463,7 +2467,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>RET-H</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2475,22 +2479,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2500,17 +2504,17 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>805579089</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>ROWING</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2520,7 +2524,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2532,24 +2536,24 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.391419</v>
+        <v>-58.451835</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.605543</v>
+        <v>-34.562646</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>CEN-E</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2561,22 +2565,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5731</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>RIOBAMBA 659</t>
+          <t>MAZA 181</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2586,7 +2590,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>807215439</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2596,7 +2600,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2618,10 +2622,10 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.394118</v>
+        <v>-58.416477</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.601416</v>
+        <v>-34.61303</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -2635,7 +2639,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>CLI-I</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2647,22 +2651,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>6076</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>MATHEU 727</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2672,19 +2676,15 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>ICD31456940</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
-        </is>
-      </c>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2704,24 +2704,24 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.451835</v>
+        <v>-58.400169</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.562646</v>
+        <v>-34.617784</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>CEN-N</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2733,22 +2733,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>6284</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>6/30/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MAZA 181</t>
+          <t>CHILE 2561</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2758,7 +2758,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>807215439</t>
+          <t>807851584</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2766,11 +2766,7 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Picada</t>
-        </is>
-      </c>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2790,10 +2786,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.416477</v>
+        <v>-58.401827</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.61303</v>
+        <v>-34.617667</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2807,7 +2803,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>CLI-I</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2819,22 +2815,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6076</t>
+          <t>5999</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>8/12/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MATHEU 727</t>
+          <t>MARMOL, JOSE 228</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2844,7 +2840,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
+          <t>808918687</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2852,7 +2848,11 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Nodo TLC</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2869,13 +2869,13 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.400169</v>
+        <v>-58.425858</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.617784</v>
+        <v>-34.61629</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>CEN-N</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2901,22 +2901,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6284</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6/30/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CHILE 2561</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2926,15 +2926,19 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>807851584</t>
+          <t>ICD30508311</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr"/>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2942,26 +2946,26 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L30" t="n">
         <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.401827</v>
+        <v>-58.435017</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.617667</v>
+        <v>-34.622044</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2971,7 +2975,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2983,22 +2987,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3008,17 +3012,17 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>ICD30593982</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3028,26 +3032,26 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.425858</v>
+        <v>-58.443232</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.61629</v>
+        <v>-34.620007</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3057,7 +3061,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3069,22 +3073,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3094,17 +3098,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>809910087</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3114,26 +3118,26 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.435017</v>
+        <v>-58.442045</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.622044</v>
+        <v>-34.594303</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3143,7 +3147,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3155,22 +3159,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>7570</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>10/6/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3180,7 +3184,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -3190,7 +3194,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3205,17 +3209,17 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.443232</v>
+        <v>-58.465176</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.620007</v>
+        <v>-34.680979</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3229,7 +3233,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>PAV-U</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3241,22 +3245,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3266,7 +3270,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -3295,27 +3299,27 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.442045</v>
+        <v>-58.444996</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.594303</v>
+        <v>-34.564443</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3327,22 +3331,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3352,17 +3356,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3381,17 +3385,17 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.465176</v>
+        <v>-58.4018</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.680979</v>
+        <v>-34.590471</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3401,7 +3405,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3413,22 +3417,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>-649</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/23/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Arribeños 1438</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3438,7 +3442,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -3448,7 +3452,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3458,36 +3462,36 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.444996</v>
+        <v>-58.436262</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.564443</v>
+        <v>-34.600478</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>BLO-K</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3499,22 +3503,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5749</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3524,17 +3528,17 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3544,7 +3548,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -3553,27 +3557,27 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.4018</v>
+        <v>-58.510994</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.590471</v>
+        <v>-34.655027</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3585,22 +3589,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S01150217</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Vera 311</t>
+          <t>LAMBARE 864</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3610,17 +3614,17 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>01230602</t>
+          <t>811453866</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Traspasar Fuente</t>
+          <t>corroida</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3630,26 +3634,26 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L38" t="n">
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.436262</v>
+        <v>-58.430579</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.600478</v>
+        <v>-34.604908</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
@@ -3659,7 +3663,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>ALM-M</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3671,22 +3675,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>3875</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>1/16/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>Castelli 60</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3696,219 +3700,47 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
+          <t>traspaso propio tlc coloco columna</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.510994</v>
+        <v>-58.404691</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.655027</v>
+        <v>-34.609194</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>CLI-D</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>8043</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>1/8/2026</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>LAMBARE 864</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>811453866</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>corroida</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>Sin equipos</t>
-        </is>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L40" t="n">
-        <v>1</v>
-      </c>
-      <c r="M40" t="n">
-        <v>-58.430579</v>
-      </c>
-      <c r="N40" t="n">
-        <v>-34.604908</v>
-      </c>
-      <c r="O40" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P40" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q40" t="inlineStr">
-        <is>
-          <t>ALM-M</t>
-        </is>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>3875</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>1/16/2026</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Castelli 60</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>FIBERWORK</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>traspaso propio tlc coloco columna</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
-      <c r="L41" t="n">
-        <v>1</v>
-      </c>
-      <c r="M41" t="n">
-        <v>-58.404691</v>
-      </c>
-      <c r="N41" t="n">
-        <v>-34.609194</v>
-      </c>
-      <c r="O41" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="P41" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q41" t="inlineStr">
-        <is>
-          <t>CLI-D</t>
-        </is>
-      </c>
-      <c r="R41" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -4367,7 +4199,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4633,17 +4465,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7758</t>
+          <t>5589</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2/20/2024</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ZABALA 2844</t>
+          <t>ARCOS 1520</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -4658,7 +4490,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>780340125</t>
+          <t>799540526</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -4668,7 +4500,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>cambiar columna y emprolijar cables y cajas de empalme que se ven en las fotos</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -4678,7 +4510,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -4687,13 +4519,13 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-58.452328</v>
+        <v>-58.449125</v>
       </c>
       <c r="N4" t="n">
-        <v>-34.572196</v>
+        <v>-34.565958</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -4707,7 +4539,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ATH-Q</t>
+          <t>BLO-M</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -4719,17 +4551,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>-143</t>
+          <t>5884</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10/7/2024</t>
+          <t>11/7/2024</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CIUDAD DE LA PAZ /ALT/ 2261</t>
+          <t>OLLEROS 2952</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4744,7 +4576,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>797752816</t>
+          <t>799450967</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -4752,7 +4584,11 @@
           <t>NEW</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Terminar transferencia, retirar columna vieja</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -4772,24 +4608,24 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>-58.458864</v>
+        <v>-58.447022</v>
       </c>
       <c r="N5" t="n">
-        <v>-34.561167</v>
+        <v>-34.575873</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>COG-H</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -4801,17 +4637,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5589</t>
+          <t>4862</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>1/23/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ARCOS 1520</t>
+          <t>ARCOS 2263</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4826,7 +4662,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>799540526</t>
+          <t>802857379</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -4836,7 +4672,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -4858,14 +4694,14 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>-58.449125</v>
+        <v>-58.455082</v>
       </c>
       <c r="N6" t="n">
-        <v>-34.565958</v>
+        <v>-34.558883</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -4875,7 +4711,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>BLO-M</t>
+          <t>BLO-P</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -4887,22 +4723,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>5884</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11/7/2024</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>OLLEROS 2952</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4912,7 +4748,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>799450967</t>
+          <t>804309655</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4922,7 +4758,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Terminar transferencia, retirar columna vieja</t>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4941,13 +4777,13 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>-58.447022</v>
+        <v>-58.441405</v>
       </c>
       <c r="N7" t="n">
-        <v>-34.575873</v>
+        <v>-34.594348</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -4961,7 +4797,7 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -4973,17 +4809,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4862</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1/23/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARCOS 2263</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4998,7 +4834,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>802857379</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -5008,7 +4844,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -5027,17 +4863,17 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>-58.455082</v>
+        <v>-58.451835</v>
       </c>
       <c r="N8" t="n">
-        <v>-34.558883</v>
+        <v>-34.562646</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -5047,7 +4883,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>BLO-P</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -5059,17 +4895,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -5084,7 +4920,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>809910087</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -5094,7 +4930,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -5116,10 +4952,10 @@
         <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>-58.441405</v>
+        <v>-58.442045</v>
       </c>
       <c r="N9" t="n">
-        <v>-34.594348</v>
+        <v>-34.594303</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -5145,17 +4981,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -5170,7 +5006,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -5180,7 +5016,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -5199,13 +5035,13 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>-58.451835</v>
+        <v>-58.444996</v>
       </c>
       <c r="N10" t="n">
-        <v>-34.562646</v>
+        <v>-34.564443</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -5219,7 +5055,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -5231,17 +5067,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -5256,7 +5092,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -5266,7 +5102,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -5276,22 +5112,22 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L11" t="n">
         <v>1</v>
       </c>
       <c r="M11" t="n">
-        <v>-58.442045</v>
+        <v>-58.436262</v>
       </c>
       <c r="N11" t="n">
-        <v>-34.594303</v>
+        <v>-34.600478</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -5305,182 +5141,10 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>-649</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>10/23/2025</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Arribeños 1438</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Picada</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>-58.444996</v>
-      </c>
-      <c r="N12" t="n">
-        <v>-34.564443</v>
-      </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>BLO-K</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>S01150217</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>10/29/2025</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Vera 311</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>01230602</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Traspasar Fuente</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>Fuente Teco</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>1</v>
-      </c>
-      <c r="M13" t="n">
-        <v>-58.436262</v>
-      </c>
-      <c r="N13" t="n">
-        <v>-34.600478</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>CLI-O</t>
-        </is>
-      </c>
-      <c r="R13" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-19 12:31:59)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -11,8 +11,8 @@
     <sheet name="PEBCOM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="NEW" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="FIBERWORK" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="INGEME" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Optical_Power" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Optical_Power" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="INGEME" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ROWING" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R39"/>
+  <dimension ref="A1:R40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1103,22 +1103,22 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>5589</t>
+          <t>4426</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12/31/2023</t>
+          <t>12/19/2024</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ARCOS 1520</t>
+          <t>LORA, FELIX 27</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1128,17 +1128,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>799540526</t>
+          <t>801768138</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Traspaso de redes y retiro de columna TLC ya traspaso el nodo</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1157,27 +1157,27 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9" t="n">
-        <v>-58.449125</v>
+        <v>-58.443626</v>
       </c>
       <c r="N9" t="n">
-        <v>-34.565958</v>
+        <v>-34.621032</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>BLO-M</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1189,17 +1189,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>5884</t>
+          <t>5589</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>11/7/2024</t>
+          <t>12/31/2023</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>OLLEROS 2952</t>
+          <t>ARCOS 1520</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1214,7 +1214,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>799450967</t>
+          <t>799540526</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1224,7 +1224,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Terminar transferencia, retirar columna vieja</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1246,24 +1246,24 @@
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>-58.447022</v>
+        <v>-58.449125</v>
       </c>
       <c r="N10" t="n">
-        <v>-34.575873</v>
+        <v>-34.565958</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>ATH-P</t>
+          <t>BLO-M</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
@@ -1275,22 +1275,22 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>5884</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>12/21/2024</t>
+          <t>11/7/2024</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>MERCEDES 254</t>
+          <t>OLLEROS 2952</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1300,17 +1300,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>799450967</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Terminar transferencia, retirar columna vieja</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1329,54 +1329,54 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>-58.484232</v>
+        <v>-58.447022</v>
       </c>
       <c r="N11" t="n">
-        <v>-34.631431</v>
+        <v>-34.575873</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>ATH-P</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4579</t>
+          <t>4082</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1/9/2025</t>
+          <t>12/21/2024</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>PASCO 10</t>
+          <t>MERCEDES 254</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1386,17 +1386,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>802438793</t>
+          <t>801901755</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>PIcada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1411,58 +1411,58 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L12" t="n">
         <v>1</v>
       </c>
       <c r="M12" t="n">
-        <v>-58.397512</v>
+        <v>-58.484232</v>
       </c>
       <c r="N12" t="n">
-        <v>-34.609923</v>
+        <v>-34.631431</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>CEN-G</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4528</t>
+          <t>4579</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>1/16/2025</t>
+          <t>1/9/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BARCO CENTENERA DEL 545</t>
+          <t>PASCO 10</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>802774521</t>
+          <t>802438793</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>PIcada</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1492,26 +1492,26 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L13" t="n">
         <v>1</v>
       </c>
       <c r="M13" t="n">
-        <v>-58.440625</v>
+        <v>-58.397512</v>
       </c>
       <c r="N13" t="n">
-        <v>-34.625499</v>
+        <v>-34.609923</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>PCH-C</t>
+          <t>CEN-G</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
@@ -1533,22 +1533,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4680</t>
+          <t>4528</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>1/22/2025</t>
+          <t>1/16/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>CUENCA 3345</t>
+          <t>BARCO CENTENERA DEL 545</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1558,17 +1558,17 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>802774521</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1590,24 +1590,24 @@
         <v>1</v>
       </c>
       <c r="M14" t="n">
-        <v>-58.496935</v>
+        <v>-58.440625</v>
       </c>
       <c r="N14" t="n">
-        <v>-34.599084</v>
+        <v>-34.625499</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>PCH-C</t>
         </is>
       </c>
       <c r="R14" t="inlineStr">
@@ -1619,22 +1619,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4862</t>
+          <t>4680</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>1/23/2025</t>
+          <t>1/22/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ARCOS 2263</t>
+          <t>CUENCA 3345</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1644,17 +1644,17 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>802857379</t>
+          <t>802843289</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1673,17 +1673,17 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M15" t="n">
-        <v>-58.455082</v>
+        <v>-58.496935</v>
       </c>
       <c r="N15" t="n">
-        <v>-34.558883</v>
+        <v>-34.599084</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1693,7 +1693,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>BLO-P</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R15" t="inlineStr">
@@ -1705,22 +1705,22 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4696</t>
+          <t>4862</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2/10/2025</t>
+          <t>1/23/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>YERBAL 489</t>
+          <t>ARCOS 2263</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1730,17 +1730,17 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>803607520</t>
+          <t>802857379</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Desmonte de columna ya traspasaron nodo</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1759,27 +1759,27 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>-58.438053</v>
+        <v>-58.455082</v>
       </c>
       <c r="N16" t="n">
-        <v>-34.617481</v>
+        <v>-34.558883</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Saavedra</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>BLO-P</t>
         </is>
       </c>
       <c r="R16" t="inlineStr">
@@ -1791,17 +1791,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>4696</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2/14/2025</t>
+          <t>2/10/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHACO 195</t>
+          <t>YERBAL 489</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>803607699</t>
+          <t>803607520</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Desmontar columna personal propio traspaso nodo</t>
+          <t>Desmonte de columna ya traspasaron nodo</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1848,10 +1848,10 @@
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.431522</v>
+        <v>-58.438053</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.617523</v>
+        <v>-34.617481</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1877,22 +1877,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>3/13/2025</t>
+          <t>2/14/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>TANDIL 4746</t>
+          <t>CHACO 195</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1902,17 +1902,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>803983204</t>
+          <t>803607699</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Desmontar columna personal propio traspaso nodo</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1922,36 +1922,36 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.487666</v>
+        <v>-58.431522</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.649704</v>
+        <v>-34.617523</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>PAV-N</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1963,22 +1963,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>3/13/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>TANDIL 4746</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1988,17 +1988,17 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>803983204</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2008,36 +2008,36 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.441405</v>
+        <v>-58.487666</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.594348</v>
+        <v>-34.649704</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PAV-N</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2049,7 +2049,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2074,17 +2074,17 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>804309801</t>
+          <t>804309655</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2106,14 +2106,14 @@
         <v>1</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.483821</v>
+        <v>-58.441405</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.677698</v>
+        <v>-34.594348</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2135,22 +2135,22 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5657</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>4/23/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>COCHABAMBA 2207</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2160,17 +2160,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>804309801</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2189,17 +2189,17 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.396135</v>
+        <v>-58.483821</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.624285</v>
+        <v>-34.677698</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2221,17 +2221,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5682</t>
+          <t>5657</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>4/23/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>República Bolivariana de Venezuela 2701</t>
+          <t>COCHABAMBA 2207</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>805507294</t>
+          <t>804903806</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2266,26 +2266,26 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.404913</v>
+        <v>-58.396135</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.615857</v>
+        <v>-34.624285</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2307,22 +2307,22 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>5682</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>4/29/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>República Bolivariana de Venezuela 2701</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2332,17 +2332,17 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>805579089</t>
+          <t>805507294</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>ROWING</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2352,26 +2352,26 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L23" t="n">
         <v>1</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.391419</v>
+        <v>-58.404913</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.605543</v>
+        <v>-34.615857</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CEN-E</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2393,7 +2393,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5731</t>
+          <t>5708</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>RIOBAMBA 659</t>
+          <t>SARMIENTO 1741</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2418,17 +2418,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>805579089</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>ROWING</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
+          <t>Pendiente de traspaso nodo y fuente</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2438,7 +2438,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2450,14 +2450,14 @@
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.394118</v>
+        <v>-58.391419</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.601416</v>
+        <v>-34.605543</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>CEN-E</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2479,22 +2479,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>5731</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>RIOBAMBA 659</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2504,17 +2504,17 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>805579188</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2536,24 +2536,24 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.451835</v>
+        <v>-58.394118</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.562646</v>
+        <v>-34.601416</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>RET-H</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2565,22 +2565,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>MAZA 181</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2590,17 +2590,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>807215439</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2622,24 +2622,24 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.416477</v>
+        <v>-58.451835</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.61303</v>
+        <v>-34.562646</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>CLI-I</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2651,22 +2651,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>6076</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MATHEU 727</t>
+          <t>MAZA 181</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
+          <t>807215439</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2684,7 +2684,11 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Picada</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2692,7 +2696,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Nodo TLC</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -2704,10 +2708,10 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.400169</v>
+        <v>-58.416477</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.617784</v>
+        <v>-34.61303</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
@@ -2721,7 +2725,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>CEN-N</t>
+          <t>CLI-I</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2733,17 +2737,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6284</t>
+          <t>6076</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6/30/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CHILE 2561</t>
+          <t>MATHEU 727</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2758,7 +2762,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>807851584</t>
+          <t>ICD31456940</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2774,7 +2778,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2786,10 +2790,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.401827</v>
+        <v>-58.400169</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.617667</v>
+        <v>-34.617784</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2803,7 +2807,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CEN-N</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2815,22 +2819,22 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>6284</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>6/30/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>CHILE 2561</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -2840,7 +2844,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>807851584</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2848,11 +2852,7 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2869,13 +2869,13 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.425858</v>
+        <v>-58.401827</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.61629</v>
+        <v>-34.617667</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2889,7 +2889,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2901,22 +2901,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>5999</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>8/12/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>MARMOL, JOSE 228</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2926,17 +2926,17 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>808918687</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2951,21 +2951,21 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.435017</v>
+        <v>-58.425858</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.622044</v>
+        <v>-34.61629</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2987,17 +2987,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -3012,7 +3012,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>ICD30508311</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -3022,7 +3022,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -3044,10 +3044,10 @@
         <v>1</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.443232</v>
+        <v>-58.435017</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.620007</v>
+        <v>-34.622044</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
@@ -3061,7 +3061,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3073,22 +3073,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3098,17 +3098,17 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>ICD30593982</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3123,21 +3123,21 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L32" t="n">
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.442045</v>
+        <v>-58.443232</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.594303</v>
+        <v>-34.620007</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3159,22 +3159,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>7570</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>10/6/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3184,17 +3184,17 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>809910087</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3216,14 +3216,14 @@
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.465176</v>
+        <v>-58.442045</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.680979</v>
+        <v>-34.594303</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>PAV-U</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3741,6 +3741,92 @@
         </is>
       </c>
       <c r="R39" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>S00552343</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2/23/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>DESCALZI, NICOLAS 5582</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Pendiente ADM OT GxC</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L40" t="n">
+        <v>1</v>
+      </c>
+      <c r="M40" t="n">
+        <v>-58.464382</v>
+      </c>
+      <c r="N40" t="n">
+        <v>-34.683083</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -6361,7 +6447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6459,22 +6545,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4082</t>
+          <t>4426</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12/21/2024</t>
+          <t>12/19/2024</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MERCEDES 254</t>
+          <t>LORA, FELIX 27</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -6484,17 +6570,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>801901755</t>
+          <t>801768138</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Traspaso de redes y retiro de columna TLC ya traspaso el nodo</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -6504,7 +6590,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -6516,51 +6602,51 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>-58.484232</v>
+        <v>-58.443626</v>
       </c>
       <c r="N2" t="n">
-        <v>-34.631431</v>
+        <v>-34.621032</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>DEV-L</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>ARATO-25058.PO.2DEV</t>
+          <t>Fuera de Poligono OVL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4680</t>
+          <t>4696</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1/22/2025</t>
+          <t>2/10/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CUENCA 3345</t>
+          <t>YERBAL 489</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -6570,17 +6656,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>802843289</t>
+          <t>803607520</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Desmonte de columna ya traspasaron nodo</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -6602,24 +6688,24 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>-58.496935</v>
+        <v>-58.438053</v>
       </c>
       <c r="N3" t="n">
-        <v>-34.599084</v>
+        <v>-34.617481</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>PUE-B</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -6631,22 +6717,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3/13/2025</t>
+          <t>2/14/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TANDIL 4746</t>
+          <t>CHACO 195</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6656,17 +6742,17 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>803983204</t>
+          <t>803607699</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Desmontar columna personal propio traspaso nodo</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -6676,36 +6762,36 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>-58.487666</v>
+        <v>-58.431522</v>
       </c>
       <c r="N4" t="n">
-        <v>-34.649704</v>
+        <v>-34.617523</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PAV-N</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -6717,22 +6803,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6742,17 +6828,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>804309801</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -6762,7 +6848,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -6774,27 +6860,285 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>-58.510994</v>
+        <v>-58.483821</v>
       </c>
       <c r="N5" t="n">
-        <v>-34.655027</v>
+        <v>-34.677698</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7051</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>8/26/2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MORENO, JOSE MARIA AV. 345</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ICD30508311</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-58.435017</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-34.622044</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>PCH-M</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4698</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>8/29/2025</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>REPETTO, NICOLAS, DR. 93</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ICD30593982</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-58.443232</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-34.620007</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>PCH-G</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>S00552343</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2/23/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DESCALZI, NICOLAS 5582</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Pendiente ADM OT GxC</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>-58.464382</v>
+      </c>
+      <c r="N8" t="n">
+        <v>-34.683083</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>PAV-U</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -6811,7 +7155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6909,22 +7253,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>4696</t>
+          <t>4082</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2/10/2025</t>
+          <t>12/21/2024</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>YERBAL 489</t>
+          <t>MERCEDES 254</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -6934,17 +7278,17 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>803607520</t>
+          <t>801901755</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Desmonte de columna ya traspasaron nodo</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -6966,51 +7310,51 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>-58.438053</v>
+        <v>-58.484232</v>
       </c>
       <c r="N2" t="n">
-        <v>-34.617481</v>
+        <v>-34.631431</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>DEV-L</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>Fuera de Poligono OVL</t>
+          <t>ARATO-25058.PO.2DEV</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>4680</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2/14/2025</t>
+          <t>1/22/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CHACO 195</t>
+          <t>CUENCA 3345</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>11</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -7020,17 +7364,17 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>803607699</t>
+          <t>802843289</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Desmontar columna personal propio traspaso nodo</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7052,24 +7396,24 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>-58.431522</v>
+        <v>-58.496935</v>
       </c>
       <c r="N3" t="n">
-        <v>-34.617523</v>
+        <v>-34.599084</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>PUE-B</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -7081,22 +7425,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>3/13/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>TANDIL 4746</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -7106,12 +7450,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>804309801</t>
+          <t>803983204</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -7126,36 +7470,36 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-58.483821</v>
+        <v>-58.487666</v>
       </c>
       <c r="N4" t="n">
-        <v>-34.677698</v>
+        <v>-34.649704</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>PAV-N</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -7167,22 +7511,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7192,17 +7536,17 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -7212,211 +7556,39 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L5" t="n">
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>-58.435017</v>
+        <v>-58.510994</v>
       </c>
       <c r="N5" t="n">
-        <v>-34.622044</v>
+        <v>-34.655027</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>4698</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>8/29/2025</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>ICD30593982</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="L6" t="n">
-        <v>1</v>
-      </c>
-      <c r="M6" t="n">
-        <v>-58.443232</v>
-      </c>
-      <c r="N6" t="n">
-        <v>-34.620007</v>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>PCH-G</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>7570</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>10/6/2025</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>VILLEGAS, CONRADO, GRAL. 5402</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>CAMBIAR COLUMNA</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L7" t="n">
-        <v>1</v>
-      </c>
-      <c r="M7" t="n">
-        <v>-58.465176</v>
-      </c>
-      <c r="N7" t="n">
-        <v>-34.680979</v>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Boedo</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>PAV-U</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-25 11:01:36)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -2079,7 +2079,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -3189,7 +3189,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3447,7 +3447,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4285,7 +4285,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4809,22 +4809,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4834,7 +4834,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -4844,7 +4844,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -4866,24 +4866,24 @@
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>-58.441405</v>
+        <v>-58.451835</v>
       </c>
       <c r="N7" t="n">
-        <v>-34.594348</v>
+        <v>-34.562646</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -4895,17 +4895,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -4930,7 +4930,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -4949,13 +4949,13 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>-58.451835</v>
+        <v>-58.444996</v>
       </c>
       <c r="N8" t="n">
-        <v>-34.562646</v>
+        <v>-34.564443</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -4969,268 +4969,10 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2712</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>9/22/2025</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>VERA 1021</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>809910087</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Picada</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>1</v>
-      </c>
-      <c r="M9" t="n">
-        <v>-58.442045</v>
-      </c>
-      <c r="N9" t="n">
-        <v>-34.594303</v>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>VCR-H</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>-649</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>10/23/2025</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Arribeños 1438</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Pendiente ADM</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Picada</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Nodo Teco</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Pasante</t>
-        </is>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>-58.444996</v>
-      </c>
-      <c r="N10" t="n">
-        <v>-34.564443</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>BLO-K</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Fuera de Poligono OVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>S01150217</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>10/29/2025</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Vera 311</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>15</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Pendiente de Traspaso PROPIO</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>01230602</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>NEW</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Traspasar Fuente</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>Cambio</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>Fuente Teco</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Terminal</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
-      <c r="M11" t="n">
-        <v>-58.436262</v>
-      </c>
-      <c r="N11" t="n">
-        <v>-34.600478</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>CLI-O</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -7155,7 +6897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7511,22 +7253,22 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -7536,7 +7278,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>804309655</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -7546,7 +7288,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -7556,7 +7298,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -7568,27 +7310,285 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
+        <v>-58.441405</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-34.594348</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>VCR-H</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2712</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>9/22/2025</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>VERA 1021</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>809910087</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Picada</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-58.442045</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-34.594303</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>VCR-H</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>S01150217</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/29/2025</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Vera 311</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>01230602</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Traspasar Fuente</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-58.436262</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-34.600478</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>CLI-O</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>-670</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11/10/2025</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Timoteo Gordillo 1666</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>810651269</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
         <v>-58.510994</v>
       </c>
-      <c r="N5" t="n">
+      <c r="N8" t="n">
         <v>-34.655027</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Devoto</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>Capital Norte</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>PAV-J</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-07-02 12:18:53)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Traspasos.xlsx
+++ b/mapa_interactivo_Traspasos.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R40"/>
+  <dimension ref="A1:R43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1791,22 +1791,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4696</t>
+          <t>4791</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2/10/2025</t>
+          <t>1/30/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>YERBAL 489</t>
+          <t>RONDEAU 2775</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1816,17 +1816,17 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>803607520</t>
+          <t>802988219</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>ROWING</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Desmonte de columna ya traspasaron nodo</t>
+          <t>Relevar</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1848,14 +1848,14 @@
         <v>1</v>
       </c>
       <c r="M17" t="n">
-        <v>-58.438053</v>
+        <v>-58.402062</v>
       </c>
       <c r="N17" t="n">
-        <v>-34.617481</v>
+        <v>-34.635143</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1865,7 +1865,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>ALM-G</t>
+          <t>PPT-K</t>
         </is>
       </c>
       <c r="R17" t="inlineStr">
@@ -1877,17 +1877,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>4696</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2/14/2025</t>
+          <t>2/10/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CHACO 195</t>
+          <t>YERBAL 489</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>803607699</t>
+          <t>803607520</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Desmontar columna personal propio traspaso nodo</t>
+          <t>Desmonte de columna ya traspasaron nodo</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1934,10 +1934,10 @@
         <v>1</v>
       </c>
       <c r="M18" t="n">
-        <v>-58.431522</v>
+        <v>-58.438053</v>
       </c>
       <c r="N18" t="n">
-        <v>-34.617523</v>
+        <v>-34.617481</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>ALM-F</t>
+          <t>ALM-G</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
@@ -1963,22 +1963,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6029</t>
+          <t>4938</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>3/13/2025</t>
+          <t>2/14/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TANDIL 4746</t>
+          <t>CHACO 195</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1988,17 +1988,17 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>803983204</t>
+          <t>803607699</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>Desmontar columna personal propio traspaso nodo</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2008,36 +2008,36 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" t="n">
-        <v>-58.487666</v>
+        <v>-58.431522</v>
       </c>
       <c r="N19" t="n">
-        <v>-34.649704</v>
+        <v>-34.617523</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>PAV-N</t>
+          <t>ALM-F</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
@@ -2049,22 +2049,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2114</t>
+          <t>6029</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>3/27/2025</t>
+          <t>3/13/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>THAMES 649</t>
+          <t>TANDIL 4746</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2074,7 +2074,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>804309655</t>
+          <t>803983204</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2094,36 +2094,36 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>-58.441405</v>
+        <v>-58.487666</v>
       </c>
       <c r="N20" t="n">
-        <v>-34.594348</v>
+        <v>-34.649704</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PAV-N</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
@@ -2135,7 +2135,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4179</t>
+          <t>2114</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2145,12 +2145,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ZELARRAYAN 6147</t>
+          <t>THAMES 649</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2160,17 +2160,17 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>804309801</t>
+          <t>804309655</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>QAP traspaso fuente propia para posterior pasar a TLC</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2192,14 +2192,14 @@
         <v>1</v>
       </c>
       <c r="M21" t="n">
-        <v>-58.483821</v>
+        <v>-58.441405</v>
       </c>
       <c r="N21" t="n">
-        <v>-34.677698</v>
+        <v>-34.594348</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>PAV-Q</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -2221,22 +2221,22 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5657</t>
+          <t>4179</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>4/23/2025</t>
+          <t>3/27/2025</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>COCHABAMBA 2207</t>
+          <t>ZELARRAYAN 6147</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2246,17 +2246,17 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>804903806</t>
+          <t>804309801</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>picada</t>
+          <t>CAMBIAR COLUMNA</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2275,17 +2275,17 @@
         </is>
       </c>
       <c r="L22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M22" t="n">
-        <v>-58.396135</v>
+        <v>-58.483821</v>
       </c>
       <c r="N22" t="n">
-        <v>-34.624285</v>
+        <v>-34.677698</v>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>CON-C</t>
+          <t>PAV-Q</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -2307,17 +2307,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>5682</t>
+          <t>5657</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4/29/2025</t>
+          <t>4/23/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>República Bolivariana de Venezuela 2701</t>
+          <t>COCHABAMBA 2207</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>805507294</t>
+          <t>804903806</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>picada</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2352,26 +2352,26 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>-58.404913</v>
+        <v>-58.396135</v>
       </c>
       <c r="N23" t="n">
-        <v>-34.615857</v>
+        <v>-34.624285</v>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CON-C</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2393,22 +2393,22 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>5682</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>4/29/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>República Bolivariana de Venezuela 2701</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2418,17 +2418,17 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>805579089</t>
+          <t>805507294</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>ROWING</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2438,26 +2438,26 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L24" t="n">
         <v>1</v>
       </c>
       <c r="M24" t="n">
-        <v>-58.391419</v>
+        <v>-58.404913</v>
       </c>
       <c r="N24" t="n">
-        <v>-34.605543</v>
+        <v>-34.615857</v>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>CEN-E</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2479,7 +2479,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>5731</t>
+          <t>5708</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2489,12 +2489,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>RIOBAMBA 659</t>
+          <t>SARMIENTO 1741</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2504,17 +2504,17 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>805579188</t>
+          <t>805579089</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>ROWING</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
+          <t>Pendiente de traspaso nodo y fuente</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo/Fuente Teco</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2536,14 +2536,14 @@
         <v>1</v>
       </c>
       <c r="M25" t="n">
-        <v>-58.394118</v>
+        <v>-58.391419</v>
       </c>
       <c r="N25" t="n">
-        <v>-34.601416</v>
+        <v>-34.605543</v>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>RET-H</t>
+          <t>CEN-E</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2565,22 +2565,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>-405</t>
+          <t>5731</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>5/8/2025</t>
+          <t>5/1/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Arcos 1855</t>
+          <t>RIOBAMBA 659</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -2590,17 +2590,17 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>805791908</t>
+          <t>805579188</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
+          <t>Pendiente de traspaso nodo entro tambien como 7100</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2622,24 +2622,24 @@
         <v>1</v>
       </c>
       <c r="M26" t="n">
-        <v>-58.451835</v>
+        <v>-58.394118</v>
       </c>
       <c r="N26" t="n">
-        <v>-34.562646</v>
+        <v>-34.601416</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>BLO-N</t>
+          <t>RET-H</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2651,22 +2651,22 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>6004</t>
+          <t>-405</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6/5/2025</t>
+          <t>5/8/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MAZA 181</t>
+          <t>Arcos 1855</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2676,17 +2676,17 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>807215439</t>
+          <t>805791908</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>Cambiar columna 114 picada en base, posee nodo propio.&lt;br&gt;</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2708,24 +2708,24 @@
         <v>1</v>
       </c>
       <c r="M27" t="n">
-        <v>-58.416477</v>
+        <v>-58.451835</v>
       </c>
       <c r="N27" t="n">
-        <v>-34.61303</v>
+        <v>-34.562646</v>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>CLI-I</t>
+          <t>BLO-N</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2737,22 +2737,22 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6076</t>
+          <t>6004</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6/24/2025</t>
+          <t>6/5/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>MATHEU 727</t>
+          <t>MAZA 181</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -2762,7 +2762,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>ICD31456940</t>
+          <t>807215439</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2770,7 +2770,11 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Picada</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2778,7 +2782,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Nodo TLC</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2790,10 +2794,10 @@
         <v>1</v>
       </c>
       <c r="M28" t="n">
-        <v>-58.400169</v>
+        <v>-58.416477</v>
       </c>
       <c r="N28" t="n">
-        <v>-34.617784</v>
+        <v>-34.61303</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -2807,7 +2811,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>CEN-N</t>
+          <t>CLI-I</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2819,17 +2823,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6284</t>
+          <t>6076</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6/30/2025</t>
+          <t>6/24/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CHILE 2561</t>
+          <t>MATHEU 727</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2844,7 +2848,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>807851584</t>
+          <t>ICD31456940</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2860,7 +2864,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Nodo TLC</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2872,10 +2876,10 @@
         <v>1</v>
       </c>
       <c r="M29" t="n">
-        <v>-58.401827</v>
+        <v>-58.400169</v>
       </c>
       <c r="N29" t="n">
-        <v>-34.617667</v>
+        <v>-34.617784</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -2889,7 +2893,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>CEN-M</t>
+          <t>CEN-N</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">
@@ -2901,22 +2905,22 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5999</t>
+          <t>6284</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>8/12/2025</t>
+          <t>6/30/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MARMOL, JOSE 228</t>
+          <t>CHILE 2561</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2926,7 +2930,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>808918687</t>
+          <t>807851584</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2934,11 +2938,7 @@
           <t>FIBERWORK</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
-        </is>
-      </c>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>Cambio</t>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -2955,13 +2955,13 @@
         </is>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M30" t="n">
-        <v>-58.425858</v>
+        <v>-58.401827</v>
       </c>
       <c r="N30" t="n">
-        <v>-34.61629</v>
+        <v>-34.617667</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -2975,7 +2975,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>ALM-D</t>
+          <t>CEN-M</t>
         </is>
       </c>
       <c r="R30" t="inlineStr">
@@ -2987,22 +2987,22 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7051</t>
+          <t>5999</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>8/26/2025</t>
+          <t>8/12/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MORENO, JOSE MARIA AV. 345</t>
+          <t>MARMOL, JOSE 228</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -3012,17 +3012,17 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ICD30508311</t>
+          <t>808918687</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>FIBERWORK</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
+          <t>Se deriva directamente a traspaso de fuente ya que hay una columna existente</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3037,21 +3037,21 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>-58.435017</v>
+        <v>-58.425858</v>
       </c>
       <c r="N31" t="n">
-        <v>-34.622044</v>
+        <v>-34.61629</v>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Almagro</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>PCH-M</t>
+          <t>ALM-D</t>
         </is>
       </c>
       <c r="R31" t="inlineStr">
@@ -3073,17 +3073,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>4698</t>
+          <t>7051</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>8/29/2025</t>
+          <t>8/26/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>REPETTO, NICOLAS, DR. 93</t>
+          <t>MORENO, JOSE MARIA AV. 345</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -3098,7 +3098,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>ICD30593982</t>
+          <t>ICD30508311</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
+          <t>Colocar PRFV R400 para pedir traspaso de fuente</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -3118,7 +3118,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3130,10 +3130,10 @@
         <v>1</v>
       </c>
       <c r="M32" t="n">
-        <v>-58.443232</v>
+        <v>-58.435017</v>
       </c>
       <c r="N32" t="n">
-        <v>-34.620007</v>
+        <v>-34.622044</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3147,7 +3147,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>PCH-G</t>
+          <t>PCH-M</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
@@ -3159,22 +3159,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2712</t>
+          <t>4698</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>9/22/2025</t>
+          <t>8/29/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>VERA 1021</t>
+          <t>REPETTO, NICOLAS, DR. 93</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3184,17 +3184,17 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>809910087</t>
+          <t>ICD30593982</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>Optical Power</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Picada</t>
+          <t>traspasar nodo a columna nueva y pasar a retirar entro directamente con la nueva al lado</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -3209,21 +3209,21 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L33" t="n">
         <v>1</v>
       </c>
       <c r="M33" t="n">
-        <v>-58.442045</v>
+        <v>-58.443232</v>
       </c>
       <c r="N33" t="n">
-        <v>-34.594303</v>
+        <v>-34.620007</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Boedo</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
@@ -3233,7 +3233,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>VCR-H</t>
+          <t>PCH-G</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
@@ -3245,22 +3245,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>-649</t>
+          <t>2712</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>10/23/2025</t>
+          <t>9/22/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Arribeños 1438</t>
+          <t>VERA 1021</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -3270,12 +3270,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>809910087</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>NEW</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3299,27 +3299,27 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M34" t="n">
-        <v>-58.444996</v>
+        <v>-58.442045</v>
       </c>
       <c r="N34" t="n">
-        <v>-34.564443</v>
+        <v>-34.594303</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>BLO-K</t>
+          <t>VCR-H</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
@@ -3331,22 +3331,22 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5749</t>
+          <t>-649</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>10/27/2025</t>
+          <t>10/23/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
+          <t>Arribeños 1438</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -3356,17 +3356,17 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>01230434</t>
+          <t>Pendiente ADM</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>PEBCOM</t>
+          <t>NEW</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
+          <t>Picada</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -3388,24 +3388,24 @@
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>-58.4018</v>
+        <v>-58.444996</v>
       </c>
       <c r="N35" t="n">
-        <v>-34.590471</v>
+        <v>-34.564443</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>Recoleta</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>AGU-F</t>
+          <t>BLO-K</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
@@ -3417,22 +3417,22 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>S01150217</t>
+          <t>5749</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>10/29/2025</t>
+          <t>10/27/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Vera 311</t>
+          <t>ANCHORENA, TOMAS MANUEL DE, DR. 1754</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -3442,17 +3442,17 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>01230602</t>
+          <t>01230434</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>INGEME</t>
+          <t>PEBCOM</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Traspasar Fuente</t>
+          <t>Traspaso de nodo propio avisar a telecentro despues del traspaso</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -3462,26 +3462,26 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>-58.436262</v>
+        <v>-58.4018</v>
       </c>
       <c r="N36" t="n">
-        <v>-34.600478</v>
+        <v>-34.590471</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>CLI-O</t>
+          <t>AGU-F</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
@@ -3503,22 +3503,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>-670</t>
+          <t>S01150217</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>11/10/2025</t>
+          <t>10/29/2025</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Timoteo Gordillo 1666</t>
+          <t>Vera 311</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -3528,7 +3528,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>810651269</t>
+          <t>01230602</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
+          <t>Traspasar Fuente</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -3548,36 +3548,36 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Sin equipos</t>
+          <t>Fuente Teco</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Pasante</t>
+          <t>Terminal</t>
         </is>
       </c>
       <c r="L37" t="n">
         <v>1</v>
       </c>
       <c r="M37" t="n">
-        <v>-58.510994</v>
+        <v>-58.436262</v>
       </c>
       <c r="N37" t="n">
-        <v>-34.655027</v>
+        <v>-34.600478</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>PAV-J</t>
+          <t>CLI-O</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
@@ -3589,22 +3589,22 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>8043</t>
+          <t>-670</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1/8/2026</t>
+          <t>11/10/2025</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LAMBARE 864</t>
+          <t>Timoteo Gordillo 1666</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -3614,17 +3614,17 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>811453866</t>
+          <t>810651269</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>FIBERWORK</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>corroida</t>
+          <t>CAMBIAR COLUMNA Y DESPLAZAR</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3646,24 +3646,24 @@
         <v>1</v>
       </c>
       <c r="M38" t="n">
-        <v>-58.430579</v>
+        <v>-58.510994</v>
       </c>
       <c r="N38" t="n">
-        <v>-34.604908</v>
+        <v>-34.655027</v>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>Almagro</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>ALM-M</t>
+          <t>PAV-J</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
@@ -3675,22 +3675,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>3875</t>
+          <t>8043</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>1/16/2026</t>
+          <t>1/8/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Castelli 60</t>
+          <t>LAMBARE 864</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3700,7 +3700,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Pendiente ADM</t>
+          <t>811453866</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3710,20 +3710,32 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>traspaso propio tlc coloco columna</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
+          <t>corroida</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
       <c r="L39" t="n">
         <v>1</v>
       </c>
       <c r="M39" t="n">
-        <v>-58.404691</v>
+        <v>-58.430579</v>
       </c>
       <c r="N39" t="n">
-        <v>-34.609194</v>
+        <v>-34.604908</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -3737,7 +3749,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>CLI-D</t>
+          <t>ALM-M</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
@@ -3749,22 +3761,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S00552343</t>
+          <t>8066</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2/23/2026</t>
+          <t>1/14/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>DESCALZI, NICOLAS 5582</t>
+          <t>FRIAS, EUSTOQUIO, TTE. GENERAL 378</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>15</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -3774,17 +3786,17 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Pendiente ADM OT GxC</t>
+          <t>811454396</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Optical Power</t>
+          <t>INGEME</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>CAMBIAR COLUMNA</t>
+          <t>inclinada corroida</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -3794,39 +3806,285 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Nodo Teco</t>
+          <t>Sin equipos</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Terminal</t>
+          <t>Pasante</t>
         </is>
       </c>
       <c r="L40" t="n">
         <v>1</v>
       </c>
       <c r="M40" t="n">
+        <v>-58.433871</v>
+      </c>
+      <c r="N40" t="n">
+        <v>-34.601836</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>ALM-N</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>3875</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1/16/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Castelli 60</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Pendiente ADM</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>FIBERWORK</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>traspaso propio tlc coloco columna</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="n">
+        <v>1</v>
+      </c>
+      <c r="M41" t="n">
+        <v>-58.404691</v>
+      </c>
+      <c r="N41" t="n">
+        <v>-34.609194</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>CLI-D</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>8322</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2/10/2026</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ARENAL, CONCEPCION 3814</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>04279107</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>inclinada corroida</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L42" t="n">
+        <v>1</v>
+      </c>
+      <c r="M42" t="n">
+        <v>-58.447805</v>
+      </c>
+      <c r="N42" t="n">
+        <v>-34.587018</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>ATH-L</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>S00552343</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2/23/2026</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>DESCALZI, NICOLAS 5582</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Pendiente ADM OT GxC</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>CAMBIAR COLUMNA</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Terminal</t>
+        </is>
+      </c>
+      <c r="L43" t="n">
+        <v>1</v>
+      </c>
+      <c r="M43" t="n">
         <v>-58.464382</v>
       </c>
-      <c r="N40" t="n">
+      <c r="N43" t="n">
         <v>-34.683083</v>
       </c>
-      <c r="O40" t="inlineStr">
+      <c r="O43" t="inlineStr">
         <is>
           <t>Boedo</t>
         </is>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>PAV-U</t>
         </is>
       </c>
-      <c r="R40" t="inlineStr">
+      <c r="R43" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -6897,7 +7155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R8"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7589,6 +7847,178 @@
         </is>
       </c>
       <c r="R8" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>8066</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1/14/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FRIAS, EUSTOQUIO, TTE. GENERAL 378</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>811454396</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>inclinada corroida</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Sin equipos</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-58.433871</v>
+      </c>
+      <c r="N9" t="n">
+        <v>-34.601836</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>ALM-N</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8322</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2/10/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ARENAL, CONCEPCION 3814</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>04279107</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>INGEME</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>inclinada corroida</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Nodo Teco</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-58.447805</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-34.587018</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>ATH-L</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>
@@ -7605,7 +8035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7703,22 +8133,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>5708</t>
+          <t>4791</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>5/1/2025</t>
+          <t>1/30/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SARMIENTO 1741</t>
+          <t>RONDEAU 2775</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -7728,7 +8158,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>805579089</t>
+          <t>802988219</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -7738,7 +8168,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Pendiente de traspaso nodo y fuente</t>
+          <t>Relevar</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7748,7 +8178,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Nodo/Fuente Teco</t>
+          <t>Nodo Teco</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -7760,27 +8190,113 @@
         <v>1</v>
       </c>
       <c r="M2" t="n">
+        <v>-58.402062</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-34.635143</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>San Telmo</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>PPT-K</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Fuera de Poligono OVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>5708</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>5/1/2025</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>SARMIENTO 1741</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pendiente de Traspaso PROPIO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>805579089</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ROWING</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Pendiente de traspaso nodo y fuente</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Cambio</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Nodo/Fuente Teco</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Pasante</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
         <v>-58.391419</v>
       </c>
-      <c r="N2" t="n">
+      <c r="N3" t="n">
         <v>-34.605543</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>San Telmo</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>CEN-E</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Fuera de Poligono OVL</t>
         </is>

</xml_diff>